<commit_message>
fix: modified app.py structure
</commit_message>
<xml_diff>
--- a/templates/Consolidación Estados Financieros e Ingresos - Plantilla.xlsx
+++ b/templates/Consolidación Estados Financieros e Ingresos - Plantilla.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jose Gonzalez\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2C6B073-D9B6-4D15-8F5E-B776CFF27F96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40780563-218B-40B3-9B54-BB45C6796549}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="816" uniqueCount="332">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="818" uniqueCount="334">
   <si>
     <t>SALDOS INICIALES Y FINALES POR CUENTA</t>
   </si>
@@ -1025,28 +1025,35 @@
     <t>19/08</t>
   </si>
   <si>
+    <t>Total</t>
+  </si>
+  <si>
     <t>Nota: el reporte suma únicamente los valores existentes en Crédito / Abono / Valor +. Los movimientos originales permanecen sin cambios.</t>
   </si>
   <si>
-    <t>SALDO DISPONIBLE</t>
-  </si>
-  <si>
-    <t>Total</t>
+    <t>Dinero disponible</t>
+  </si>
+  <si>
+    <t>SALDO FINAL TOTAL</t>
+  </si>
+  <si>
+    <t>DINERO DISPONIBLE</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="6">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="166" formatCode="\$#,##0.00"/>
     <numFmt numFmtId="167" formatCode="0000"/>
     <numFmt numFmtId="168" formatCode="\$#,##0.00;[Red]\-\$#,##0.00"/>
     <numFmt numFmtId="169" formatCode="\Q\ #,##0.00;[Red]\(\Q\ #,##0.00\);\-"/>
+    <numFmt numFmtId="170" formatCode="\Q\ #,##0.00;[Red]\-\Q\ #,##0.00"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1143,17 +1150,36 @@
       <sz val="11"/>
       <color rgb="FF008080"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="2" tint="-0.749961851863155"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF008080"/>
+      <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
-      <sz val="15"/>
-      <color theme="2" tint="-0.749992370372631"/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1217,12 +1243,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79995117038483843"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -1241,13 +1273,28 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="4" tint="-0.249977111117893"/>
+      </left>
+      <right style="thin">
+        <color theme="4" tint="-0.249977111117893"/>
+      </right>
+      <top style="thin">
+        <color theme="4" tint="-0.249977111117893"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="-0.249977111117893"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1269,18 +1316,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1328,6 +1363,7 @@
     <xf numFmtId="169" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="169" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="169" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1344,6 +1380,24 @@
     <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="10" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="13" fillId="10" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="169" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1355,23 +1409,29 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="10" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="13" fillId="10" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="170" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="10" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1379,8 +1439,116 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="5">
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color theme="4" tint="-0.249977111117893"/>
+        </left>
+        <right style="thin">
+          <color theme="4" tint="-0.249977111117893"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color theme="4" tint="-0.249977111117893"/>
+        </vertical>
+        <horizontal style="thin">
+          <color theme="4" tint="-0.249977111117893"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color theme="4" tint="-0.249977111117893"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="-0.249977111117893"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="-0.249977111117893"/>
+        </bottom>
+        <vertical style="thin">
+          <color theme="4" tint="-0.249977111117893"/>
+        </vertical>
+        <horizontal style="thin">
+          <color theme="4" tint="-0.249977111117893"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color theme="4" tint="-0.249977111117893"/>
+        </left>
+        <right style="thin">
+          <color theme="4" tint="-0.249977111117893"/>
+        </right>
+        <top style="thin">
+          <color theme="4" tint="-0.249977111117893"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="-0.249977111117893"/>
+        </bottom>
+        <vertical style="thin">
+          <color theme="4" tint="-0.249977111117893"/>
+        </vertical>
+        <horizontal style="thin">
+          <color theme="4" tint="-0.249977111117893"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color theme="4" tint="-0.249977111117893"/>
+        </left>
+        <right style="thin">
+          <color theme="4" tint="-0.249977111117893"/>
+        </right>
+        <top style="thin">
+          <color theme="4" tint="-0.249977111117893"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="-0.249977111117893"/>
+        </bottom>
+        <vertical style="thin">
+          <color theme="4" tint="-0.249977111117893"/>
+        </vertical>
+        <horizontal style="thin">
+          <color theme="4" tint="-0.249977111117893"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color theme="4" tint="-0.249977111117893"/>
+        </right>
+        <top style="thin">
+          <color theme="4" tint="-0.249977111117893"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="-0.249977111117893"/>
+        </bottom>
+        <vertical style="thin">
+          <color theme="4" tint="-0.249977111117893"/>
+        </vertical>
+        <horizontal style="thin">
+          <color theme="4" tint="-0.249977111117893"/>
+        </horizontal>
+      </border>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FF008080"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1584,7 +1752,7 @@
           <c:smooth val="1"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-6594-47E3-8145-010E8EFD41FC}"/>
+              <c16:uniqueId val="{00000000-BDED-475D-8FDA-8AF14A29C274}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1812,7 +1980,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-92AC-41A0-8F27-E22BB8285E16}"/>
+              <c16:uniqueId val="{00000000-93C6-4152-9E78-A22C24564008}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1946,12 +2114,12 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="SaldosPorCuenta" displayName="SaldosPorCuenta" ref="A4:D12" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="SaldosPorCuenta" displayName="SaldosPorCuenta" ref="A4:D12" totalsRowShown="0" headerRowDxfId="0">
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Banco"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Cuenta"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Saldo inicial "/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Saldo final "/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Banco" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Cuenta" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Saldo inicial " dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Saldo final " dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2152,7 +2320,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:F200"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.33203125" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="27.44140625" style="8" customWidth="1"/>
@@ -2161,152 +2329,745 @@
     <col min="5" max="16384" width="10.33203125" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="20.85" customHeight="1">
-      <c r="A1" s="38" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
-    </row>
-    <row r="2" spans="1:4" ht="22.35" customHeight="1">
-      <c r="A2" s="40" t="s">
+    <row r="1" spans="1:6" ht="16.649999999999999" customHeight="1">
+      <c r="A1" s="35" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+    </row>
+    <row r="2" spans="1:6" ht="17.850000000000001" customHeight="1">
+      <c r="A2" s="37" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="39"/>
-      <c r="C2" s="39"/>
-      <c r="D2" s="39"/>
-    </row>
-    <row r="4" spans="1:4" ht="24" customHeight="1">
-      <c r="A4" s="9" t="s">
+      <c r="B2" s="36"/>
+      <c r="C2" s="36"/>
+      <c r="D2" s="36"/>
+    </row>
+    <row r="4" spans="1:6" ht="19.2" customHeight="1">
+      <c r="A4" s="54" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="54" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="54" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="D4" s="54" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" ht="16.05" customHeight="1">
-      <c r="A5" s="10" t="s">
+      <c r="E4" s="55" t="s">
+        <v>331</v>
+      </c>
+      <c r="F4" s="55"/>
+    </row>
+    <row r="5" spans="1:6" ht="12.75" customHeight="1">
+      <c r="A5" s="56" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="57" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="12">
+      <c r="C5" s="58">
         <v>76663.7</v>
       </c>
-      <c r="D5" s="12">
+      <c r="D5" s="58">
         <v>71075.34</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" ht="16.05" customHeight="1">
-      <c r="A6" s="10" t="s">
+      <c r="E5" s="59"/>
+      <c r="F5" s="59"/>
+    </row>
+    <row r="6" spans="1:6" ht="12.75" customHeight="1">
+      <c r="A6" s="56" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="57" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="12">
+      <c r="C6" s="58">
         <v>14148.75</v>
       </c>
-      <c r="D6" s="12">
+      <c r="D6" s="58">
         <v>21941.21</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" ht="16.05" customHeight="1">
-      <c r="A7" s="10" t="s">
+      <c r="E6" s="59"/>
+      <c r="F6" s="59"/>
+    </row>
+    <row r="7" spans="1:6" ht="12.75" customHeight="1">
+      <c r="A7" s="56" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="57" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="12">
+      <c r="C7" s="58">
         <v>33171.599999999999</v>
       </c>
-      <c r="D7" s="12">
+      <c r="D7" s="58">
         <v>28319.18</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" ht="16.05" customHeight="1">
-      <c r="A8" s="10" t="s">
+      <c r="E7" s="59"/>
+      <c r="F7" s="59"/>
+    </row>
+    <row r="8" spans="1:6" ht="12.75" customHeight="1">
+      <c r="A8" s="56" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="57" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="12">
+      <c r="C8" s="58">
         <v>9086.82</v>
       </c>
-      <c r="D8" s="12">
+      <c r="D8" s="58">
         <v>6003.86</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" ht="16.05" customHeight="1">
-      <c r="A9" s="10" t="s">
+      <c r="E8" s="59"/>
+      <c r="F8" s="59"/>
+    </row>
+    <row r="9" spans="1:6" ht="12.75" customHeight="1">
+      <c r="A9" s="56" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="B9" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="12">
+      <c r="C9" s="58">
         <v>80183.38</v>
       </c>
-      <c r="D9" s="12">
+      <c r="D9" s="58">
         <v>81910.289999999994</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" ht="16.05" customHeight="1">
-      <c r="A10" s="10" t="s">
+      <c r="E9" s="59"/>
+      <c r="F9" s="59"/>
+    </row>
+    <row r="10" spans="1:6" ht="12.75" customHeight="1">
+      <c r="A10" s="56" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="57" t="s">
         <v>15</v>
       </c>
-      <c r="C10" s="12">
+      <c r="C10" s="58">
         <v>51799.49</v>
       </c>
-      <c r="D10" s="12">
+      <c r="D10" s="58">
         <v>33700.51</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" ht="16.05" customHeight="1">
-      <c r="A11" s="10" t="s">
+      <c r="E10" s="59"/>
+      <c r="F10" s="59"/>
+    </row>
+    <row r="11" spans="1:6" ht="12.75" customHeight="1">
+      <c r="A11" s="56" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="11" t="s">
+      <c r="B11" s="57" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="12">
+      <c r="C11" s="58">
         <v>38443.89</v>
       </c>
-      <c r="D11" s="12">
+      <c r="D11" s="58">
         <v>25869.5</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" ht="16.05" customHeight="1">
-      <c r="A12" s="10" t="s">
+      <c r="E11" s="59"/>
+      <c r="F11" s="59"/>
+    </row>
+    <row r="12" spans="1:6" ht="12.75" customHeight="1">
+      <c r="A12" s="56" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="11" t="s">
+      <c r="B12" s="57" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="12">
+      <c r="C12" s="58">
         <v>31.71</v>
       </c>
-      <c r="D12" s="12">
+      <c r="D12" s="58">
         <v>125.63</v>
       </c>
+      <c r="E12" s="59"/>
+      <c r="F12" s="59"/>
+    </row>
+    <row r="13" spans="1:6" ht="14.4">
+      <c r="E13" s="34"/>
+    </row>
+    <row r="14" spans="1:6" ht="14.4">
+      <c r="E14" s="34"/>
+    </row>
+    <row r="15" spans="1:6" ht="14.4">
+      <c r="E15" s="34"/>
+    </row>
+    <row r="16" spans="1:6" ht="14.4">
+      <c r="E16" s="34"/>
+    </row>
+    <row r="17" spans="5:5" ht="14.4">
+      <c r="E17" s="34"/>
+    </row>
+    <row r="18" spans="5:5" ht="14.4">
+      <c r="E18" s="34"/>
+    </row>
+    <row r="19" spans="5:5" ht="14.4">
+      <c r="E19" s="34"/>
+    </row>
+    <row r="20" spans="5:5" ht="14.4">
+      <c r="E20" s="34"/>
+    </row>
+    <row r="21" spans="5:5" ht="14.4">
+      <c r="E21" s="34"/>
+    </row>
+    <row r="22" spans="5:5" ht="14.4">
+      <c r="E22" s="34"/>
+    </row>
+    <row r="23" spans="5:5" ht="14.4">
+      <c r="E23" s="34"/>
+    </row>
+    <row r="24" spans="5:5" ht="14.4">
+      <c r="E24" s="34"/>
+    </row>
+    <row r="25" spans="5:5" ht="14.4">
+      <c r="E25" s="34"/>
+    </row>
+    <row r="26" spans="5:5" ht="14.4">
+      <c r="E26" s="34"/>
+    </row>
+    <row r="27" spans="5:5" ht="14.4">
+      <c r="E27" s="34"/>
+    </row>
+    <row r="28" spans="5:5" ht="14.4">
+      <c r="E28" s="34"/>
+    </row>
+    <row r="29" spans="5:5" ht="14.4">
+      <c r="E29" s="34"/>
+    </row>
+    <row r="30" spans="5:5" ht="14.4">
+      <c r="E30" s="34"/>
+    </row>
+    <row r="31" spans="5:5" ht="14.4">
+      <c r="E31" s="34"/>
+    </row>
+    <row r="32" spans="5:5" ht="14.4">
+      <c r="E32" s="34"/>
+    </row>
+    <row r="33" spans="5:5" ht="14.4">
+      <c r="E33" s="34"/>
+    </row>
+    <row r="34" spans="5:5" ht="14.4">
+      <c r="E34" s="34"/>
+    </row>
+    <row r="35" spans="5:5" ht="14.4">
+      <c r="E35" s="34"/>
+    </row>
+    <row r="36" spans="5:5" ht="14.4">
+      <c r="E36" s="34"/>
+    </row>
+    <row r="37" spans="5:5" ht="14.4">
+      <c r="E37" s="34"/>
+    </row>
+    <row r="38" spans="5:5" ht="14.4">
+      <c r="E38" s="34"/>
+    </row>
+    <row r="39" spans="5:5" ht="14.4">
+      <c r="E39" s="34"/>
+    </row>
+    <row r="40" spans="5:5" ht="14.4">
+      <c r="E40" s="34"/>
+    </row>
+    <row r="41" spans="5:5" ht="14.4">
+      <c r="E41" s="34"/>
+    </row>
+    <row r="42" spans="5:5" ht="14.4">
+      <c r="E42" s="34"/>
+    </row>
+    <row r="43" spans="5:5" ht="14.4">
+      <c r="E43" s="34"/>
+    </row>
+    <row r="44" spans="5:5" ht="14.4">
+      <c r="E44" s="34"/>
+    </row>
+    <row r="45" spans="5:5" ht="14.4">
+      <c r="E45" s="34"/>
+    </row>
+    <row r="46" spans="5:5" ht="14.4">
+      <c r="E46" s="34"/>
+    </row>
+    <row r="47" spans="5:5" ht="14.4">
+      <c r="E47" s="34"/>
+    </row>
+    <row r="48" spans="5:5" ht="14.4">
+      <c r="E48" s="34"/>
+    </row>
+    <row r="49" spans="5:5" ht="14.4">
+      <c r="E49" s="34"/>
+    </row>
+    <row r="50" spans="5:5" ht="14.4">
+      <c r="E50" s="34"/>
+    </row>
+    <row r="51" spans="5:5" ht="14.4">
+      <c r="E51" s="34"/>
+    </row>
+    <row r="52" spans="5:5" ht="14.4">
+      <c r="E52" s="34"/>
+    </row>
+    <row r="53" spans="5:5" ht="14.4">
+      <c r="E53" s="34"/>
+    </row>
+    <row r="54" spans="5:5" ht="14.4">
+      <c r="E54" s="34"/>
+    </row>
+    <row r="55" spans="5:5" ht="14.4">
+      <c r="E55" s="34"/>
+    </row>
+    <row r="56" spans="5:5" ht="14.4">
+      <c r="E56" s="34"/>
+    </row>
+    <row r="57" spans="5:5" ht="14.4">
+      <c r="E57" s="34"/>
+    </row>
+    <row r="58" spans="5:5" ht="14.4">
+      <c r="E58" s="34"/>
+    </row>
+    <row r="59" spans="5:5" ht="14.4">
+      <c r="E59" s="34"/>
+    </row>
+    <row r="60" spans="5:5" ht="14.4">
+      <c r="E60" s="34"/>
+    </row>
+    <row r="61" spans="5:5" ht="14.4">
+      <c r="E61" s="34"/>
+    </row>
+    <row r="62" spans="5:5" ht="14.4">
+      <c r="E62" s="34"/>
+    </row>
+    <row r="63" spans="5:5" ht="14.4">
+      <c r="E63" s="34"/>
+    </row>
+    <row r="64" spans="5:5" ht="14.4">
+      <c r="E64" s="34"/>
+    </row>
+    <row r="65" spans="5:5" ht="14.4">
+      <c r="E65" s="34"/>
+    </row>
+    <row r="66" spans="5:5" ht="14.4">
+      <c r="E66" s="34"/>
+    </row>
+    <row r="67" spans="5:5" ht="14.4">
+      <c r="E67" s="34"/>
+    </row>
+    <row r="68" spans="5:5" ht="14.4">
+      <c r="E68" s="34"/>
+    </row>
+    <row r="69" spans="5:5" ht="14.4">
+      <c r="E69" s="34"/>
+    </row>
+    <row r="70" spans="5:5" ht="14.4">
+      <c r="E70" s="34"/>
+    </row>
+    <row r="71" spans="5:5" ht="14.4">
+      <c r="E71" s="34"/>
+    </row>
+    <row r="72" spans="5:5" ht="14.4">
+      <c r="E72" s="34"/>
+    </row>
+    <row r="73" spans="5:5" ht="14.4">
+      <c r="E73" s="34"/>
+    </row>
+    <row r="74" spans="5:5" ht="14.4">
+      <c r="E74" s="34"/>
+    </row>
+    <row r="75" spans="5:5" ht="14.4">
+      <c r="E75" s="34"/>
+    </row>
+    <row r="76" spans="5:5" ht="14.4">
+      <c r="E76" s="34"/>
+    </row>
+    <row r="77" spans="5:5" ht="14.4">
+      <c r="E77" s="34"/>
+    </row>
+    <row r="78" spans="5:5" ht="14.4">
+      <c r="E78" s="34"/>
+    </row>
+    <row r="79" spans="5:5" ht="14.4">
+      <c r="E79" s="34"/>
+    </row>
+    <row r="80" spans="5:5" ht="14.4">
+      <c r="E80" s="34"/>
+    </row>
+    <row r="81" spans="5:5" ht="14.4">
+      <c r="E81" s="34"/>
+    </row>
+    <row r="82" spans="5:5" ht="14.4">
+      <c r="E82" s="34"/>
+    </row>
+    <row r="83" spans="5:5" ht="14.4">
+      <c r="E83" s="34"/>
+    </row>
+    <row r="84" spans="5:5" ht="14.4">
+      <c r="E84" s="34"/>
+    </row>
+    <row r="85" spans="5:5" ht="14.4">
+      <c r="E85" s="34"/>
+    </row>
+    <row r="86" spans="5:5" ht="14.4">
+      <c r="E86" s="34"/>
+    </row>
+    <row r="87" spans="5:5" ht="14.4">
+      <c r="E87" s="34"/>
+    </row>
+    <row r="88" spans="5:5" ht="14.4">
+      <c r="E88" s="34"/>
+    </row>
+    <row r="89" spans="5:5" ht="14.4">
+      <c r="E89" s="34"/>
+    </row>
+    <row r="90" spans="5:5" ht="14.4">
+      <c r="E90" s="34"/>
+    </row>
+    <row r="91" spans="5:5" ht="14.4">
+      <c r="E91" s="34"/>
+    </row>
+    <row r="92" spans="5:5" ht="14.4">
+      <c r="E92" s="34"/>
+    </row>
+    <row r="93" spans="5:5" ht="14.4">
+      <c r="E93" s="34"/>
+    </row>
+    <row r="94" spans="5:5" ht="14.4">
+      <c r="E94" s="34"/>
+    </row>
+    <row r="95" spans="5:5" ht="14.4">
+      <c r="E95" s="34"/>
+    </row>
+    <row r="96" spans="5:5" ht="14.4">
+      <c r="E96" s="34"/>
+    </row>
+    <row r="97" spans="5:5" ht="14.4">
+      <c r="E97" s="34"/>
+    </row>
+    <row r="98" spans="5:5" ht="14.4">
+      <c r="E98" s="34"/>
+    </row>
+    <row r="99" spans="5:5" ht="14.4">
+      <c r="E99" s="34"/>
+    </row>
+    <row r="100" spans="5:5" ht="14.4">
+      <c r="E100" s="34"/>
+    </row>
+    <row r="101" spans="5:5" ht="14.4">
+      <c r="E101" s="34"/>
+    </row>
+    <row r="102" spans="5:5" ht="14.4">
+      <c r="E102" s="34"/>
+    </row>
+    <row r="103" spans="5:5" ht="14.4">
+      <c r="E103" s="34"/>
+    </row>
+    <row r="104" spans="5:5" ht="14.4">
+      <c r="E104" s="34"/>
+    </row>
+    <row r="105" spans="5:5" ht="14.4">
+      <c r="E105" s="34"/>
+    </row>
+    <row r="106" spans="5:5" ht="14.4">
+      <c r="E106" s="34"/>
+    </row>
+    <row r="107" spans="5:5" ht="14.4">
+      <c r="E107" s="34"/>
+    </row>
+    <row r="108" spans="5:5" ht="14.4">
+      <c r="E108" s="34"/>
+    </row>
+    <row r="109" spans="5:5" ht="14.4">
+      <c r="E109" s="34"/>
+    </row>
+    <row r="110" spans="5:5" ht="14.4">
+      <c r="E110" s="34"/>
+    </row>
+    <row r="111" spans="5:5" ht="14.4">
+      <c r="E111" s="34"/>
+    </row>
+    <row r="112" spans="5:5" ht="14.4">
+      <c r="E112" s="34"/>
+    </row>
+    <row r="113" spans="5:5" ht="14.4">
+      <c r="E113" s="34"/>
+    </row>
+    <row r="114" spans="5:5" ht="14.4">
+      <c r="E114" s="34"/>
+    </row>
+    <row r="115" spans="5:5" ht="14.4">
+      <c r="E115" s="34"/>
+    </row>
+    <row r="116" spans="5:5" ht="14.4">
+      <c r="E116" s="34"/>
+    </row>
+    <row r="117" spans="5:5" ht="14.4">
+      <c r="E117" s="34"/>
+    </row>
+    <row r="118" spans="5:5" ht="14.4">
+      <c r="E118" s="34"/>
+    </row>
+    <row r="119" spans="5:5" ht="14.4">
+      <c r="E119" s="34"/>
+    </row>
+    <row r="120" spans="5:5" ht="14.4">
+      <c r="E120" s="34"/>
+    </row>
+    <row r="121" spans="5:5" ht="14.4">
+      <c r="E121" s="34"/>
+    </row>
+    <row r="122" spans="5:5" ht="14.4">
+      <c r="E122" s="34"/>
+    </row>
+    <row r="123" spans="5:5" ht="14.4">
+      <c r="E123" s="34"/>
+    </row>
+    <row r="124" spans="5:5" ht="14.4">
+      <c r="E124" s="34"/>
+    </row>
+    <row r="125" spans="5:5" ht="14.4">
+      <c r="E125" s="34"/>
+    </row>
+    <row r="126" spans="5:5" ht="14.4">
+      <c r="E126" s="34"/>
+    </row>
+    <row r="127" spans="5:5" ht="14.4">
+      <c r="E127" s="34"/>
+    </row>
+    <row r="128" spans="5:5" ht="14.4">
+      <c r="E128" s="34"/>
+    </row>
+    <row r="129" spans="5:5" ht="14.4">
+      <c r="E129" s="34"/>
+    </row>
+    <row r="130" spans="5:5" ht="14.4">
+      <c r="E130" s="34"/>
+    </row>
+    <row r="131" spans="5:5" ht="14.4">
+      <c r="E131" s="34"/>
+    </row>
+    <row r="132" spans="5:5" ht="14.4">
+      <c r="E132" s="34"/>
+    </row>
+    <row r="133" spans="5:5" ht="14.4">
+      <c r="E133" s="34"/>
+    </row>
+    <row r="134" spans="5:5" ht="14.4">
+      <c r="E134" s="34"/>
+    </row>
+    <row r="135" spans="5:5" ht="14.4">
+      <c r="E135" s="34"/>
+    </row>
+    <row r="136" spans="5:5" ht="14.4">
+      <c r="E136" s="34"/>
+    </row>
+    <row r="137" spans="5:5" ht="14.4">
+      <c r="E137" s="34"/>
+    </row>
+    <row r="138" spans="5:5" ht="14.4">
+      <c r="E138" s="34"/>
+    </row>
+    <row r="139" spans="5:5" ht="14.4">
+      <c r="E139" s="34"/>
+    </row>
+    <row r="140" spans="5:5" ht="14.4">
+      <c r="E140" s="34"/>
+    </row>
+    <row r="141" spans="5:5" ht="14.4">
+      <c r="E141" s="34"/>
+    </row>
+    <row r="142" spans="5:5" ht="14.4">
+      <c r="E142" s="34"/>
+    </row>
+    <row r="143" spans="5:5" ht="14.4">
+      <c r="E143" s="34"/>
+    </row>
+    <row r="144" spans="5:5" ht="14.4">
+      <c r="E144" s="34"/>
+    </row>
+    <row r="145" spans="5:5" ht="14.4">
+      <c r="E145" s="34"/>
+    </row>
+    <row r="146" spans="5:5" ht="14.4">
+      <c r="E146" s="34"/>
+    </row>
+    <row r="147" spans="5:5" ht="14.4">
+      <c r="E147" s="34"/>
+    </row>
+    <row r="148" spans="5:5" ht="14.4">
+      <c r="E148" s="34"/>
+    </row>
+    <row r="149" spans="5:5" ht="14.4">
+      <c r="E149" s="34"/>
+    </row>
+    <row r="150" spans="5:5" ht="14.4">
+      <c r="E150" s="34"/>
+    </row>
+    <row r="151" spans="5:5" ht="14.4">
+      <c r="E151" s="34"/>
+    </row>
+    <row r="152" spans="5:5" ht="14.4">
+      <c r="E152" s="34"/>
+    </row>
+    <row r="153" spans="5:5" ht="14.4">
+      <c r="E153" s="34"/>
+    </row>
+    <row r="154" spans="5:5" ht="14.4">
+      <c r="E154" s="34"/>
+    </row>
+    <row r="155" spans="5:5" ht="14.4">
+      <c r="E155" s="34"/>
+    </row>
+    <row r="156" spans="5:5" ht="14.4">
+      <c r="E156" s="34"/>
+    </row>
+    <row r="157" spans="5:5" ht="14.4">
+      <c r="E157" s="34"/>
+    </row>
+    <row r="158" spans="5:5" ht="14.4">
+      <c r="E158" s="34"/>
+    </row>
+    <row r="159" spans="5:5" ht="14.4">
+      <c r="E159" s="34"/>
+    </row>
+    <row r="160" spans="5:5" ht="14.4">
+      <c r="E160" s="34"/>
+    </row>
+    <row r="161" spans="5:5" ht="14.4">
+      <c r="E161" s="34"/>
+    </row>
+    <row r="162" spans="5:5" ht="14.4">
+      <c r="E162" s="34"/>
+    </row>
+    <row r="163" spans="5:5" ht="14.4">
+      <c r="E163" s="34"/>
+    </row>
+    <row r="164" spans="5:5" ht="14.4">
+      <c r="E164" s="34"/>
+    </row>
+    <row r="165" spans="5:5" ht="14.4">
+      <c r="E165" s="34"/>
+    </row>
+    <row r="166" spans="5:5" ht="14.4">
+      <c r="E166" s="34"/>
+    </row>
+    <row r="167" spans="5:5" ht="14.4">
+      <c r="E167" s="34"/>
+    </row>
+    <row r="168" spans="5:5" ht="14.4">
+      <c r="E168" s="34"/>
+    </row>
+    <row r="169" spans="5:5" ht="14.4">
+      <c r="E169" s="34"/>
+    </row>
+    <row r="170" spans="5:5" ht="14.4">
+      <c r="E170" s="34"/>
+    </row>
+    <row r="171" spans="5:5" ht="14.4">
+      <c r="E171" s="34"/>
+    </row>
+    <row r="172" spans="5:5" ht="14.4">
+      <c r="E172" s="34"/>
+    </row>
+    <row r="173" spans="5:5" ht="14.4">
+      <c r="E173" s="34"/>
+    </row>
+    <row r="174" spans="5:5" ht="14.4">
+      <c r="E174" s="34"/>
+    </row>
+    <row r="175" spans="5:5" ht="14.4">
+      <c r="E175" s="34"/>
+    </row>
+    <row r="176" spans="5:5" ht="14.4">
+      <c r="E176" s="34"/>
+    </row>
+    <row r="177" spans="5:5" ht="14.4">
+      <c r="E177" s="34"/>
+    </row>
+    <row r="178" spans="5:5" ht="14.4">
+      <c r="E178" s="34"/>
+    </row>
+    <row r="179" spans="5:5" ht="14.4">
+      <c r="E179" s="34"/>
+    </row>
+    <row r="180" spans="5:5" ht="14.4">
+      <c r="E180" s="34"/>
+    </row>
+    <row r="181" spans="5:5" ht="14.4">
+      <c r="E181" s="34"/>
+    </row>
+    <row r="182" spans="5:5" ht="14.4">
+      <c r="E182" s="34"/>
+    </row>
+    <row r="183" spans="5:5" ht="14.4">
+      <c r="E183" s="34"/>
+    </row>
+    <row r="184" spans="5:5" ht="14.4">
+      <c r="E184" s="34"/>
+    </row>
+    <row r="185" spans="5:5" ht="14.4">
+      <c r="E185" s="34"/>
+    </row>
+    <row r="186" spans="5:5" ht="14.4">
+      <c r="E186" s="34"/>
+    </row>
+    <row r="187" spans="5:5" ht="14.4">
+      <c r="E187" s="34"/>
+    </row>
+    <row r="188" spans="5:5" ht="14.4">
+      <c r="E188" s="34"/>
+    </row>
+    <row r="189" spans="5:5" ht="14.4">
+      <c r="E189" s="34"/>
+    </row>
+    <row r="190" spans="5:5" ht="14.4">
+      <c r="E190" s="34"/>
+    </row>
+    <row r="191" spans="5:5" ht="14.4">
+      <c r="E191" s="34"/>
+    </row>
+    <row r="192" spans="5:5" ht="14.4">
+      <c r="E192" s="34"/>
+    </row>
+    <row r="193" spans="5:5" ht="14.4">
+      <c r="E193" s="34"/>
+    </row>
+    <row r="194" spans="5:5" ht="14.4">
+      <c r="E194" s="34"/>
+    </row>
+    <row r="195" spans="5:5" ht="14.4">
+      <c r="E195" s="34"/>
+    </row>
+    <row r="196" spans="5:5" ht="14.4">
+      <c r="E196" s="34"/>
+    </row>
+    <row r="197" spans="5:5" ht="14.4">
+      <c r="E197" s="34"/>
+    </row>
+    <row r="198" spans="5:5" ht="14.4">
+      <c r="E198" s="34"/>
+    </row>
+    <row r="199" spans="5:5" ht="14.4">
+      <c r="E199" s="34"/>
+    </row>
+    <row r="200" spans="5:5" ht="14.4">
+      <c r="E200" s="34"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="11">
+    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="E11:F11"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="E6:F6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -2332,7 +3093,7 @@
     <col min="10" max="16384" width="10.33203125" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="27.15" customHeight="1">
+    <row r="1" spans="1:8" ht="21.75" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -7133,620 +7894,620 @@
     <col min="12" max="16384" width="10.33203125" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="24" customHeight="1">
-      <c r="A1" s="41" t="s">
+    <row r="1" spans="1:11" ht="19.2" customHeight="1">
+      <c r="A1" s="38" t="s">
         <v>286</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
-      <c r="E1" s="39"/>
-      <c r="F1" s="39"/>
-      <c r="G1" s="39"/>
-      <c r="H1" s="39"/>
-      <c r="I1" s="39"/>
-      <c r="J1" s="39"/>
-      <c r="K1" s="39"/>
-    </row>
-    <row r="2" spans="1:11" ht="22.35" customHeight="1">
-      <c r="A2" s="42" t="s">
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
+      <c r="G1" s="36"/>
+      <c r="H1" s="36"/>
+      <c r="I1" s="36"/>
+      <c r="J1" s="36"/>
+      <c r="K1" s="36"/>
+    </row>
+    <row r="2" spans="1:11" ht="17.850000000000001" customHeight="1">
+      <c r="A2" s="39" t="s">
         <v>287</v>
       </c>
-      <c r="B2" s="39"/>
-      <c r="C2" s="39"/>
-      <c r="D2" s="39"/>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="39"/>
-      <c r="H2" s="39"/>
-      <c r="I2" s="39"/>
-      <c r="J2" s="39"/>
-      <c r="K2" s="39"/>
+      <c r="B2" s="36"/>
+      <c r="C2" s="36"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
+      <c r="G2" s="36"/>
+      <c r="H2" s="36"/>
+      <c r="I2" s="36"/>
+      <c r="J2" s="36"/>
+      <c r="K2" s="36"/>
     </row>
     <row r="3" spans="1:11">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="9" t="s">
         <v>288</v>
       </c>
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="43" t="s">
+      <c r="C3" s="40" t="s">
         <v>289</v>
       </c>
-      <c r="D3" s="39"/>
-      <c r="E3" s="43" t="s">
+      <c r="D3" s="36"/>
+      <c r="E3" s="40" t="s">
         <v>130</v>
       </c>
-      <c r="F3" s="39"/>
-      <c r="G3" s="13" t="s">
+      <c r="F3" s="36"/>
+      <c r="G3" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="H3" s="43" t="s">
+      <c r="H3" s="40" t="s">
         <v>241</v>
       </c>
-      <c r="I3" s="39"/>
-      <c r="J3" s="13"/>
-      <c r="K3" s="13"/>
-    </row>
-    <row r="4" spans="1:11" ht="20.85" customHeight="1">
-      <c r="A4" s="14" t="s">
+      <c r="I3" s="36"/>
+      <c r="J3" s="9"/>
+      <c r="K3" s="9"/>
+    </row>
+    <row r="4" spans="1:11" ht="16.649999999999999" customHeight="1">
+      <c r="A4" s="10" t="s">
         <v>290</v>
       </c>
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="15" t="s">
+      <c r="C4" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="E4" s="15" t="s">
+      <c r="E4" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="F4" s="15" t="s">
+      <c r="F4" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="G4" s="15" t="s">
+      <c r="G4" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="H4" s="15" t="s">
+      <c r="H4" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="I4" s="15" t="s">
+      <c r="I4" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="J4" s="14" t="s">
+      <c r="J4" s="10" t="s">
         <v>291</v>
       </c>
-      <c r="K4" s="14" t="s">
+      <c r="K4" s="10" t="s">
         <v>292</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="16.8" customHeight="1">
-      <c r="A5" s="16">
+    <row r="5" spans="1:11" ht="13.35" customHeight="1">
+      <c r="A5" s="12">
         <v>46235</v>
       </c>
-      <c r="B5" s="17">
+      <c r="B5" s="13">
         <v>124.3</v>
       </c>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17">
+      <c r="C5" s="13"/>
+      <c r="D5" s="13">
         <v>176.16</v>
       </c>
-      <c r="E5" s="17">
+      <c r="E5" s="13">
         <v>1015.83</v>
       </c>
-      <c r="F5" s="17">
+      <c r="F5" s="13">
         <v>8400</v>
       </c>
-      <c r="G5" s="17"/>
-      <c r="H5" s="17"/>
-      <c r="I5" s="17"/>
-      <c r="J5" s="18">
+      <c r="G5" s="13"/>
+      <c r="H5" s="13"/>
+      <c r="I5" s="13"/>
+      <c r="J5" s="14">
         <v>9716.2900000000009</v>
       </c>
-      <c r="K5" s="19">
+      <c r="K5" s="15">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="16.8" customHeight="1">
-      <c r="A6" s="20">
+    <row r="6" spans="1:11" ht="13.35" customHeight="1">
+      <c r="A6" s="16">
         <v>46236</v>
       </c>
-      <c r="B6" s="21"/>
-      <c r="C6" s="21"/>
-      <c r="D6" s="21"/>
-      <c r="E6" s="21"/>
-      <c r="F6" s="21"/>
-      <c r="G6" s="21"/>
-      <c r="H6" s="21"/>
-      <c r="I6" s="21"/>
-      <c r="J6" s="18">
-        <v>0</v>
-      </c>
-      <c r="K6" s="22">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" ht="16.8" customHeight="1">
-      <c r="A7" s="16">
+      <c r="B6" s="17"/>
+      <c r="C6" s="17"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="17"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="17"/>
+      <c r="H6" s="17"/>
+      <c r="I6" s="17"/>
+      <c r="J6" s="14">
+        <v>0</v>
+      </c>
+      <c r="K6" s="18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="13.35" customHeight="1">
+      <c r="A7" s="12">
         <v>46237</v>
       </c>
-      <c r="B7" s="17">
+      <c r="B7" s="13">
         <v>333.35</v>
       </c>
-      <c r="C7" s="17"/>
-      <c r="D7" s="17">
+      <c r="C7" s="13"/>
+      <c r="D7" s="13">
         <v>508.93</v>
       </c>
-      <c r="E7" s="17"/>
-      <c r="F7" s="17">
+      <c r="E7" s="13"/>
+      <c r="F7" s="13">
         <v>940.8</v>
       </c>
-      <c r="G7" s="17">
+      <c r="G7" s="13">
         <v>560.48</v>
       </c>
-      <c r="H7" s="17"/>
-      <c r="I7" s="17"/>
-      <c r="J7" s="18">
+      <c r="H7" s="13"/>
+      <c r="I7" s="13"/>
+      <c r="J7" s="14">
         <v>2343.56</v>
       </c>
-      <c r="K7" s="19">
+      <c r="K7" s="15">
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="16.8" customHeight="1">
-      <c r="A8" s="20">
+    <row r="8" spans="1:11" ht="13.35" customHeight="1">
+      <c r="A8" s="16">
         <v>46238</v>
       </c>
-      <c r="B8" s="21">
+      <c r="B8" s="17">
         <v>1929.79</v>
       </c>
-      <c r="C8" s="21">
+      <c r="C8" s="17">
         <v>985.6</v>
       </c>
-      <c r="D8" s="21">
+      <c r="D8" s="17">
         <v>160</v>
       </c>
-      <c r="E8" s="21">
+      <c r="E8" s="17">
         <v>827.16</v>
       </c>
-      <c r="F8" s="21">
+      <c r="F8" s="17">
         <v>211.31</v>
       </c>
-      <c r="G8" s="21">
+      <c r="G8" s="17">
         <v>57.63</v>
       </c>
-      <c r="H8" s="21">
+      <c r="H8" s="17">
         <v>124.3</v>
       </c>
-      <c r="I8" s="21"/>
-      <c r="J8" s="18">
+      <c r="I8" s="17"/>
+      <c r="J8" s="14">
         <v>4295.79</v>
       </c>
-      <c r="K8" s="22">
+      <c r="K8" s="18">
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="16.8" customHeight="1">
-      <c r="A9" s="16">
+    <row r="9" spans="1:11" ht="13.35" customHeight="1">
+      <c r="A9" s="12">
         <v>46239</v>
       </c>
-      <c r="B9" s="17">
+      <c r="B9" s="13">
         <v>197.75</v>
       </c>
-      <c r="C9" s="17"/>
-      <c r="D9" s="17">
+      <c r="C9" s="13"/>
+      <c r="D9" s="13">
         <v>100</v>
       </c>
-      <c r="E9" s="17">
+      <c r="E9" s="13">
         <v>45.2</v>
       </c>
-      <c r="F9" s="17">
+      <c r="F9" s="13">
         <v>824.9</v>
       </c>
-      <c r="G9" s="17"/>
-      <c r="H9" s="17">
+      <c r="G9" s="13"/>
+      <c r="H9" s="13">
         <v>335.61</v>
       </c>
-      <c r="I9" s="17"/>
-      <c r="J9" s="18">
+      <c r="I9" s="13"/>
+      <c r="J9" s="14">
         <v>1503.46</v>
       </c>
-      <c r="K9" s="19">
+      <c r="K9" s="15">
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="16.8" customHeight="1">
-      <c r="A10" s="20">
+    <row r="10" spans="1:11" ht="13.35" customHeight="1">
+      <c r="A10" s="16">
         <v>46240</v>
       </c>
-      <c r="B10" s="21">
+      <c r="B10" s="17">
         <v>622.82000000000005</v>
       </c>
-      <c r="C10" s="21"/>
-      <c r="D10" s="21"/>
-      <c r="E10" s="21"/>
-      <c r="F10" s="21"/>
-      <c r="G10" s="21"/>
-      <c r="H10" s="21"/>
-      <c r="I10" s="21"/>
-      <c r="J10" s="18">
+      <c r="C10" s="17"/>
+      <c r="D10" s="17"/>
+      <c r="E10" s="17"/>
+      <c r="F10" s="17"/>
+      <c r="G10" s="17"/>
+      <c r="H10" s="17"/>
+      <c r="I10" s="17"/>
+      <c r="J10" s="14">
         <v>622.82000000000005</v>
       </c>
-      <c r="K10" s="22">
+      <c r="K10" s="18">
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="16.8" customHeight="1">
-      <c r="A11" s="16">
+    <row r="11" spans="1:11" ht="13.35" customHeight="1">
+      <c r="A11" s="12">
         <v>46241</v>
       </c>
-      <c r="B11" s="17">
+      <c r="B11" s="13">
         <v>1115.8800000000001</v>
       </c>
-      <c r="C11" s="17">
+      <c r="C11" s="13">
         <v>67.8</v>
       </c>
-      <c r="D11" s="17">
+      <c r="D11" s="13">
         <v>461.98</v>
       </c>
-      <c r="E11" s="17">
+      <c r="E11" s="13">
         <v>1021.92</v>
       </c>
-      <c r="F11" s="17"/>
-      <c r="G11" s="17">
+      <c r="F11" s="13"/>
+      <c r="G11" s="13">
         <v>76.84</v>
       </c>
-      <c r="H11" s="17"/>
-      <c r="I11" s="17">
+      <c r="H11" s="13"/>
+      <c r="I11" s="13">
         <v>22.02</v>
       </c>
-      <c r="J11" s="18">
+      <c r="J11" s="14">
         <v>2766.44</v>
       </c>
-      <c r="K11" s="19">
+      <c r="K11" s="15">
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="16.8" customHeight="1">
-      <c r="A12" s="20">
+    <row r="12" spans="1:11" ht="13.35" customHeight="1">
+      <c r="A12" s="16">
         <v>46242</v>
       </c>
-      <c r="B12" s="21"/>
-      <c r="C12" s="21"/>
-      <c r="D12" s="21"/>
-      <c r="E12" s="21">
+      <c r="B12" s="17"/>
+      <c r="C12" s="17"/>
+      <c r="D12" s="17"/>
+      <c r="E12" s="17">
         <v>814.73</v>
       </c>
-      <c r="F12" s="21"/>
-      <c r="G12" s="21"/>
-      <c r="H12" s="21"/>
-      <c r="I12" s="21"/>
-      <c r="J12" s="18">
+      <c r="F12" s="17"/>
+      <c r="G12" s="17"/>
+      <c r="H12" s="17"/>
+      <c r="I12" s="17"/>
+      <c r="J12" s="14">
         <v>814.73</v>
       </c>
-      <c r="K12" s="22">
+      <c r="K12" s="18">
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="16.8" customHeight="1">
-      <c r="A13" s="16">
+    <row r="13" spans="1:11" ht="13.35" customHeight="1">
+      <c r="A13" s="12">
         <v>46243</v>
       </c>
-      <c r="B13" s="17"/>
-      <c r="C13" s="17"/>
-      <c r="D13" s="17"/>
-      <c r="E13" s="17"/>
-      <c r="F13" s="17"/>
-      <c r="G13" s="17"/>
-      <c r="H13" s="17"/>
-      <c r="I13" s="17"/>
-      <c r="J13" s="18">
-        <v>0</v>
-      </c>
-      <c r="K13" s="19">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" ht="16.8" customHeight="1">
-      <c r="A14" s="20">
+      <c r="B13" s="13"/>
+      <c r="C13" s="13"/>
+      <c r="D13" s="13"/>
+      <c r="E13" s="13"/>
+      <c r="F13" s="13"/>
+      <c r="G13" s="13"/>
+      <c r="H13" s="13"/>
+      <c r="I13" s="13"/>
+      <c r="J13" s="14">
+        <v>0</v>
+      </c>
+      <c r="K13" s="15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="13.35" customHeight="1">
+      <c r="A14" s="16">
         <v>46244</v>
       </c>
-      <c r="B14" s="21">
+      <c r="B14" s="17">
         <v>716.42</v>
       </c>
-      <c r="C14" s="21">
+      <c r="C14" s="17">
         <v>113.14</v>
       </c>
-      <c r="D14" s="21">
+      <c r="D14" s="17">
         <v>267.26</v>
       </c>
-      <c r="E14" s="21"/>
-      <c r="F14" s="21">
+      <c r="E14" s="17"/>
+      <c r="F14" s="17">
         <v>911.91</v>
       </c>
-      <c r="G14" s="21">
+      <c r="G14" s="17">
         <v>554.83000000000004</v>
       </c>
-      <c r="H14" s="21">
+      <c r="H14" s="17">
         <v>192.1</v>
       </c>
-      <c r="I14" s="21">
+      <c r="I14" s="17">
         <v>79.89</v>
       </c>
-      <c r="J14" s="18">
+      <c r="J14" s="14">
         <v>2835.55</v>
       </c>
-      <c r="K14" s="22">
+      <c r="K14" s="18">
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="16.8" customHeight="1">
-      <c r="A15" s="16">
+    <row r="15" spans="1:11" ht="13.35" customHeight="1">
+      <c r="A15" s="12">
         <v>46245</v>
       </c>
-      <c r="B15" s="17">
+      <c r="B15" s="13">
         <v>904</v>
       </c>
-      <c r="C15" s="17">
+      <c r="C15" s="13">
         <v>372.9</v>
       </c>
-      <c r="D15" s="17">
+      <c r="D15" s="13">
         <v>604.79999999999995</v>
       </c>
-      <c r="E15" s="17">
-        <v>0</v>
-      </c>
-      <c r="F15" s="17">
+      <c r="E15" s="13">
+        <v>0</v>
+      </c>
+      <c r="F15" s="13">
         <v>225.25</v>
       </c>
-      <c r="G15" s="17">
+      <c r="G15" s="13">
         <v>552.16</v>
       </c>
-      <c r="H15" s="17">
+      <c r="H15" s="13">
         <v>30319</v>
       </c>
-      <c r="I15" s="17"/>
-      <c r="J15" s="18">
+      <c r="I15" s="13"/>
+      <c r="J15" s="14">
         <v>32978.11</v>
       </c>
-      <c r="K15" s="19">
+      <c r="K15" s="15">
         <v>6</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="16.8" customHeight="1">
-      <c r="A16" s="20">
+    <row r="16" spans="1:11" ht="13.35" customHeight="1">
+      <c r="A16" s="16">
         <v>46246</v>
       </c>
-      <c r="B16" s="21">
+      <c r="B16" s="17">
         <v>6110.3</v>
       </c>
-      <c r="C16" s="21"/>
-      <c r="D16" s="21">
+      <c r="C16" s="17"/>
+      <c r="D16" s="17">
         <v>729.98</v>
       </c>
-      <c r="E16" s="21">
+      <c r="E16" s="17">
         <v>640.59</v>
       </c>
-      <c r="F16" s="21">
+      <c r="F16" s="17">
         <v>281.29000000000002</v>
       </c>
-      <c r="G16" s="21">
+      <c r="G16" s="17">
         <v>56.5</v>
       </c>
-      <c r="H16" s="21">
+      <c r="H16" s="17">
         <v>544.59</v>
       </c>
-      <c r="I16" s="21"/>
-      <c r="J16" s="18">
+      <c r="I16" s="17"/>
+      <c r="J16" s="14">
         <v>8363.25</v>
       </c>
-      <c r="K16" s="22">
+      <c r="K16" s="18">
         <v>6</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="16.8" customHeight="1">
-      <c r="A17" s="16">
+    <row r="17" spans="1:11" ht="13.35" customHeight="1">
+      <c r="A17" s="12">
         <v>46247</v>
       </c>
-      <c r="B17" s="17">
+      <c r="B17" s="13">
         <v>604.86</v>
       </c>
-      <c r="C17" s="17">
+      <c r="C17" s="13">
         <v>1.38</v>
       </c>
-      <c r="D17" s="17"/>
-      <c r="E17" s="17">
+      <c r="D17" s="13"/>
+      <c r="E17" s="13">
         <v>169.3</v>
       </c>
-      <c r="F17" s="17">
+      <c r="F17" s="13">
         <v>564.08000000000004</v>
       </c>
-      <c r="G17" s="17">
+      <c r="G17" s="13">
         <v>1681.24</v>
       </c>
-      <c r="H17" s="17">
+      <c r="H17" s="13">
         <v>216.96</v>
       </c>
-      <c r="I17" s="17"/>
-      <c r="J17" s="18">
+      <c r="I17" s="13"/>
+      <c r="J17" s="14">
         <v>3237.82</v>
       </c>
-      <c r="K17" s="19">
+      <c r="K17" s="15">
         <v>6</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="16.8" customHeight="1">
-      <c r="A18" s="20">
+    <row r="18" spans="1:11" ht="13.35" customHeight="1">
+      <c r="A18" s="16">
         <v>46248</v>
       </c>
-      <c r="B18" s="21">
+      <c r="B18" s="17">
         <v>9077.44</v>
       </c>
-      <c r="C18" s="21">
+      <c r="C18" s="17">
         <v>66.67</v>
       </c>
-      <c r="D18" s="21">
+      <c r="D18" s="17">
         <v>25.99</v>
       </c>
-      <c r="E18" s="21">
+      <c r="E18" s="17">
         <v>1893.46</v>
       </c>
-      <c r="F18" s="21">
-        <v>0</v>
-      </c>
-      <c r="G18" s="21">
+      <c r="F18" s="17">
+        <v>0</v>
+      </c>
+      <c r="G18" s="17">
         <v>335.61</v>
       </c>
-      <c r="H18" s="21">
-        <v>0</v>
-      </c>
-      <c r="I18" s="21"/>
-      <c r="J18" s="18">
+      <c r="H18" s="17">
+        <v>0</v>
+      </c>
+      <c r="I18" s="17"/>
+      <c r="J18" s="14">
         <v>11399.17</v>
       </c>
-      <c r="K18" s="22">
+      <c r="K18" s="18">
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="16.8" customHeight="1">
-      <c r="A19" s="16">
+    <row r="19" spans="1:11" ht="13.35" customHeight="1">
+      <c r="A19" s="12">
         <v>46249</v>
       </c>
-      <c r="B19" s="17"/>
-      <c r="C19" s="17"/>
-      <c r="D19" s="17">
+      <c r="B19" s="13"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13">
         <v>532.23</v>
       </c>
-      <c r="E19" s="17">
+      <c r="E19" s="13">
         <v>40.99</v>
       </c>
-      <c r="F19" s="17">
+      <c r="F19" s="13">
         <v>84.75</v>
       </c>
-      <c r="G19" s="17"/>
-      <c r="H19" s="17">
+      <c r="G19" s="13"/>
+      <c r="H19" s="13">
         <v>244.08</v>
       </c>
-      <c r="I19" s="17"/>
-      <c r="J19" s="18">
+      <c r="I19" s="13"/>
+      <c r="J19" s="14">
         <v>902.05</v>
       </c>
-      <c r="K19" s="19">
+      <c r="K19" s="15">
         <v>4</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="16.8" customHeight="1">
-      <c r="A20" s="20">
+    <row r="20" spans="1:11" ht="13.35" customHeight="1">
+      <c r="A20" s="16">
         <v>46250</v>
       </c>
-      <c r="B20" s="21">
+      <c r="B20" s="17">
         <v>282.5</v>
       </c>
-      <c r="C20" s="21"/>
-      <c r="D20" s="21"/>
-      <c r="E20" s="21">
+      <c r="C20" s="17"/>
+      <c r="D20" s="17"/>
+      <c r="E20" s="17">
         <v>237.34</v>
       </c>
-      <c r="F20" s="21"/>
-      <c r="G20" s="21"/>
-      <c r="H20" s="21"/>
-      <c r="I20" s="21"/>
-      <c r="J20" s="18">
+      <c r="F20" s="17"/>
+      <c r="G20" s="17"/>
+      <c r="H20" s="17"/>
+      <c r="I20" s="17"/>
+      <c r="J20" s="14">
         <v>519.84</v>
       </c>
-      <c r="K20" s="22">
+      <c r="K20" s="18">
         <v>2</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="16.8" customHeight="1">
-      <c r="A21" s="16">
+    <row r="21" spans="1:11" ht="13.35" customHeight="1">
+      <c r="A21" s="12">
         <v>46251</v>
       </c>
-      <c r="B21" s="17">
+      <c r="B21" s="13">
         <v>387.59</v>
       </c>
-      <c r="C21" s="17">
+      <c r="C21" s="13">
         <v>21.47</v>
       </c>
-      <c r="D21" s="17">
+      <c r="D21" s="13">
         <v>793.26</v>
       </c>
-      <c r="E21" s="17"/>
-      <c r="F21" s="17">
+      <c r="E21" s="13"/>
+      <c r="F21" s="13">
         <v>637.25</v>
       </c>
-      <c r="G21" s="17">
+      <c r="G21" s="13">
         <v>966.05</v>
       </c>
-      <c r="H21" s="17">
+      <c r="H21" s="13">
         <v>728.06</v>
       </c>
-      <c r="I21" s="17"/>
-      <c r="J21" s="18">
+      <c r="I21" s="13"/>
+      <c r="J21" s="14">
         <v>3533.68</v>
       </c>
-      <c r="K21" s="19">
+      <c r="K21" s="15">
         <v>6</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="16.8" customHeight="1">
-      <c r="A22" s="20">
+    <row r="22" spans="1:11" ht="13.35" customHeight="1">
+      <c r="A22" s="16">
         <v>46252</v>
       </c>
-      <c r="B22" s="21">
+      <c r="B22" s="17">
         <v>1671.29</v>
       </c>
-      <c r="C22" s="21">
+      <c r="C22" s="17">
         <v>6163.5</v>
       </c>
-      <c r="D22" s="21">
+      <c r="D22" s="17">
         <v>339</v>
       </c>
-      <c r="E22" s="21">
+      <c r="E22" s="17">
         <v>307.38</v>
       </c>
-      <c r="F22" s="21"/>
-      <c r="G22" s="21">
+      <c r="F22" s="17"/>
+      <c r="G22" s="17">
         <v>310.24</v>
       </c>
-      <c r="H22" s="21"/>
-      <c r="I22" s="21"/>
-      <c r="J22" s="18">
+      <c r="H22" s="17"/>
+      <c r="I22" s="17"/>
+      <c r="J22" s="14">
         <v>8791.41</v>
       </c>
-      <c r="K22" s="22">
+      <c r="K22" s="18">
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="16.8" customHeight="1">
-      <c r="A23" s="16">
+    <row r="23" spans="1:11" ht="13.35" customHeight="1">
+      <c r="A23" s="12">
         <v>46253</v>
       </c>
-      <c r="B23" s="17">
+      <c r="B23" s="13">
         <v>371.77</v>
       </c>
-      <c r="C23" s="17"/>
-      <c r="D23" s="17">
+      <c r="C23" s="13"/>
+      <c r="D23" s="13">
         <v>56.5</v>
       </c>
-      <c r="E23" s="17">
+      <c r="E23" s="13">
         <v>2093.02</v>
       </c>
-      <c r="F23" s="17">
+      <c r="F23" s="13">
         <v>5251.38</v>
       </c>
-      <c r="G23" s="17">
+      <c r="G23" s="13">
         <v>485.25</v>
       </c>
-      <c r="H23" s="17"/>
-      <c r="I23" s="17"/>
-      <c r="J23" s="18">
+      <c r="H23" s="13"/>
+      <c r="I23" s="13"/>
+      <c r="J23" s="14">
         <v>8257.92</v>
       </c>
-      <c r="K23" s="19">
+      <c r="K23" s="15">
         <v>5</v>
       </c>
     </row>
@@ -7780,771 +8541,789 @@
     <col min="26" max="16384" width="10.33203125" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="25.65" customHeight="1">
-      <c r="A1" s="41" t="s">
+    <row r="1" spans="1:25" ht="20.55" customHeight="1">
+      <c r="A1" s="38" t="s">
         <v>293</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
-      <c r="E1" s="39"/>
-      <c r="F1" s="39"/>
-      <c r="G1" s="39"/>
-      <c r="H1" s="39"/>
-      <c r="X1" s="23" t="s">
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
+      <c r="G1" s="36"/>
+      <c r="H1" s="36"/>
+      <c r="X1" s="19" t="s">
         <v>290</v>
       </c>
-      <c r="Y1" s="37" t="s">
+      <c r="Y1" s="33" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="22.35" customHeight="1">
-      <c r="A2" s="42" t="s">
+    <row r="2" spans="1:25" ht="17.850000000000001" customHeight="1">
+      <c r="A2" s="39" t="s">
         <v>295</v>
       </c>
-      <c r="B2" s="39"/>
-      <c r="C2" s="39"/>
-      <c r="D2" s="39"/>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="39"/>
-      <c r="H2" s="39"/>
-      <c r="X2" s="23" t="s">
+      <c r="B2" s="36"/>
+      <c r="C2" s="36"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
+      <c r="G2" s="36"/>
+      <c r="H2" s="36"/>
+      <c r="X2" s="19" t="s">
         <v>296</v>
       </c>
-      <c r="Y2" s="37">
+      <c r="Y2" s="33">
         <f t="shared" ref="Y2:Y20" si="0">B15</f>
         <v>9716.2900000000009</v>
       </c>
     </row>
     <row r="3" spans="1:25">
-      <c r="X3" s="23" t="s">
+      <c r="X3" s="19" t="s">
         <v>297</v>
       </c>
-      <c r="Y3" s="37">
+      <c r="Y3" s="33">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:25">
-      <c r="A4" s="14" t="s">
+    <row r="4" spans="1:25" ht="12" customHeight="1">
+      <c r="A4" s="10" t="s">
         <v>298</v>
       </c>
-      <c r="B4" s="14"/>
-      <c r="C4" s="14" t="s">
+      <c r="B4" s="10"/>
+      <c r="C4" s="10" t="s">
         <v>299</v>
       </c>
-      <c r="D4" s="14"/>
-      <c r="E4" s="14" t="s">
+      <c r="D4" s="10"/>
+      <c r="E4" s="10" t="s">
         <v>300</v>
       </c>
-      <c r="F4" s="14"/>
-      <c r="G4" s="14" t="s">
+      <c r="F4" s="10"/>
+      <c r="G4" s="10" t="s">
         <v>288</v>
       </c>
-      <c r="H4" s="14"/>
-      <c r="X4" s="23" t="s">
+      <c r="H4" s="10"/>
+      <c r="X4" s="19" t="s">
         <v>301</v>
       </c>
-      <c r="Y4" s="37">
+      <c r="Y4" s="33">
         <f t="shared" si="0"/>
         <v>2343.56</v>
       </c>
     </row>
-    <row r="5" spans="1:25" ht="12" customHeight="1">
-      <c r="A5" s="49">
+    <row r="5" spans="1:25" ht="26.4" customHeight="1">
+      <c r="A5" s="44">
         <v>46235</v>
       </c>
-      <c r="B5" s="39"/>
-      <c r="C5" s="49">
+      <c r="B5" s="36"/>
+      <c r="C5" s="44">
         <v>46253</v>
       </c>
-      <c r="D5" s="39"/>
-      <c r="E5" s="50" t="s">
+      <c r="D5" s="36"/>
+      <c r="E5" s="45" t="s">
         <v>302</v>
       </c>
-      <c r="F5" s="39"/>
-      <c r="G5" s="51" t="s">
+      <c r="F5" s="36"/>
+      <c r="G5" s="46" t="s">
         <v>303</v>
       </c>
-      <c r="H5" s="39"/>
-      <c r="X5" s="23" t="s">
+      <c r="H5" s="36"/>
+      <c r="X5" s="19" t="s">
         <v>304</v>
       </c>
-      <c r="Y5" s="37">
+      <c r="Y5" s="33">
         <f t="shared" si="0"/>
         <v>4295.79</v>
       </c>
     </row>
     <row r="6" spans="1:25">
-      <c r="X6" s="23" t="s">
+      <c r="X6" s="19" t="s">
         <v>305</v>
       </c>
-      <c r="Y6" s="37">
+      <c r="Y6" s="33">
         <f t="shared" si="0"/>
         <v>1503.46</v>
       </c>
     </row>
     <row r="7" spans="1:25" ht="14.4">
-      <c r="A7" s="13" t="s">
+      <c r="A7" s="9" t="s">
         <v>306</v>
       </c>
-      <c r="B7" s="13"/>
-      <c r="C7" s="13" t="s">
+      <c r="B7" s="9"/>
+      <c r="C7" s="9" t="s">
         <v>307</v>
       </c>
-      <c r="D7" s="13"/>
-      <c r="E7" s="13" t="s">
+      <c r="D7" s="9"/>
+      <c r="E7" s="9" t="s">
         <v>308</v>
       </c>
-      <c r="F7" s="13"/>
-      <c r="G7" s="13" t="s">
+      <c r="F7" s="9"/>
+      <c r="G7" s="9" t="s">
         <v>292</v>
       </c>
-      <c r="H7" s="13"/>
-      <c r="I7" s="53" t="s">
-        <v>330</v>
-      </c>
-      <c r="J7" s="53"/>
-      <c r="X7" s="23" t="s">
+      <c r="H7" s="9"/>
+      <c r="I7" s="41" t="s">
+        <v>332</v>
+      </c>
+      <c r="J7" s="41"/>
+      <c r="K7" s="52" t="s">
+        <v>333</v>
+      </c>
+      <c r="L7" s="52"/>
+      <c r="X7" s="19" t="s">
         <v>309</v>
       </c>
-      <c r="Y7" s="37">
+      <c r="Y7" s="33">
         <f t="shared" si="0"/>
         <v>622.82000000000005</v>
       </c>
     </row>
-    <row r="8" spans="1:25" ht="15.6" customHeight="1">
-      <c r="A8" s="44">
+    <row r="8" spans="1:25" ht="16.2" customHeight="1">
+      <c r="A8" s="47">
         <f>SUM(H15:H22)</f>
         <v>102881.89</v>
       </c>
-      <c r="B8" s="45"/>
-      <c r="C8" s="44">
+      <c r="B8" s="48"/>
+      <c r="C8" s="47">
         <f>IFERROR(AVERAGEIF(H15:H22,"&gt;0"),0)</f>
         <v>12860.23625</v>
       </c>
-      <c r="D8" s="45"/>
-      <c r="E8" s="44">
+      <c r="D8" s="48"/>
+      <c r="E8" s="47">
         <f>IFERROR(MAX(H15:H22),0)</f>
         <v>32704.7</v>
       </c>
-      <c r="F8" s="45"/>
-      <c r="G8" s="46">
+      <c r="F8" s="48"/>
+      <c r="G8" s="49">
         <f>COUNTIF(H15:H22,"&gt;0")</f>
         <v>8</v>
       </c>
-      <c r="H8" s="47"/>
-      <c r="I8" s="54">
-        <f>IF($E$5&lt;&gt;"TODAS",SUMIF('SALDOS POR CUENTA'!$B$5:$B$100,$E$5,'SALDOS POR CUENTA'!$D$5:$D$100),IF($G$5&lt;&gt;"TODOS",SUMIF('SALDOS POR CUENTA'!$A$5:$A$100,"*"&amp;SUBSTITUTE(TRIM($G$5),"BANCO ","")&amp;"*",'SALDOS POR CUENTA'!$D$5:$D$100),SUM('SALDOS POR CUENTA'!$D$5:$D$100)))</f>
+      <c r="H8" s="50"/>
+      <c r="I8" s="42">
+        <f>IF($E$5&lt;&gt;"TODAS",IFERROR(SUMIF('SALDOS POR CUENTA'!$B$5:$B$200,$E$5,'SALDOS POR CUENTA'!$D$5:$D$200),0),IF($G$5&lt;&gt;"TODOS",IFERROR(SUMIF('SALDOS POR CUENTA'!$A$5:$A$200,$G$5,'SALDOS POR CUENTA'!$D$5:$D$200),0),IFERROR(SUM('SALDOS POR CUENTA'!$D$5:$D$200),0)))</f>
         <v>268945.52</v>
       </c>
-      <c r="J8" s="54"/>
-      <c r="X8" s="23" t="s">
+      <c r="J8" s="42"/>
+      <c r="K8" s="53">
+        <f>IF($E$5&lt;&gt;"TODAS",IFERROR(SUMIF('SALDOS POR CUENTA'!$B$5:$B$200,$E$5,'SALDOS POR CUENTA'!$E$5:$E$200),0),IF($G$5&lt;&gt;"TODOS",IFERROR(SUMIF('SALDOS POR CUENTA'!$A$5:$A$200,$G$5,'SALDOS POR CUENTA'!$E$5:$E$200),0),IFERROR(SUM('SALDOS POR CUENTA'!$E$5:$E$200),0)))</f>
+        <v>0</v>
+      </c>
+      <c r="L8" s="53"/>
+      <c r="X8" s="19" t="s">
         <v>310</v>
       </c>
-      <c r="Y8" s="37">
+      <c r="Y8" s="33">
         <f t="shared" si="0"/>
         <v>2766.44</v>
       </c>
     </row>
     <row r="9" spans="1:25">
-      <c r="X9" s="23" t="s">
+      <c r="X9" s="19" t="s">
         <v>311</v>
       </c>
-      <c r="Y9" s="37">
+      <c r="Y9" s="33">
         <f t="shared" si="0"/>
         <v>814.73</v>
       </c>
     </row>
-    <row r="10" spans="1:25" ht="6.45" customHeight="1">
-      <c r="A10" s="24"/>
-      <c r="B10" s="24"/>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="24"/>
-      <c r="G10" s="24"/>
-      <c r="H10" s="24"/>
-      <c r="X10" s="23" t="s">
+    <row r="10" spans="1:25" ht="5.0999999999999996" customHeight="1">
+      <c r="A10" s="20"/>
+      <c r="B10" s="20"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="20"/>
+      <c r="E10" s="20"/>
+      <c r="F10" s="20"/>
+      <c r="G10" s="20"/>
+      <c r="H10" s="20"/>
+      <c r="X10" s="19" t="s">
         <v>312</v>
       </c>
-      <c r="Y10" s="37">
+      <c r="Y10" s="33">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:25">
-      <c r="X11" s="23" t="s">
+      <c r="X11" s="19" t="s">
         <v>313</v>
       </c>
-      <c r="Y11" s="37">
+      <c r="Y11" s="33">
         <f t="shared" si="0"/>
         <v>2835.55</v>
       </c>
     </row>
     <row r="12" spans="1:25">
-      <c r="X12" s="23" t="s">
+      <c r="X12" s="19" t="s">
         <v>314</v>
       </c>
-      <c r="Y12" s="37">
+      <c r="Y12" s="33">
         <f t="shared" si="0"/>
         <v>32978.11</v>
       </c>
     </row>
-    <row r="13" spans="1:25" ht="12" customHeight="1">
-      <c r="A13" s="48" t="s">
+    <row r="13" spans="1:25" ht="9.6" customHeight="1">
+      <c r="A13" s="51" t="s">
         <v>315</v>
       </c>
-      <c r="B13" s="39"/>
-      <c r="C13" s="39"/>
-      <c r="D13" s="39"/>
-      <c r="F13" s="48" t="s">
+      <c r="B13" s="36"/>
+      <c r="C13" s="36"/>
+      <c r="D13" s="36"/>
+      <c r="F13" s="51" t="s">
         <v>316</v>
       </c>
-      <c r="G13" s="39"/>
-      <c r="H13" s="39"/>
-      <c r="X13" s="23" t="s">
+      <c r="G13" s="36"/>
+      <c r="H13" s="36"/>
+      <c r="X13" s="19" t="s">
         <v>317</v>
       </c>
-      <c r="Y13" s="37">
+      <c r="Y13" s="33">
         <f t="shared" si="0"/>
         <v>8363.25</v>
       </c>
     </row>
     <row r="14" spans="1:25">
-      <c r="A14" s="14" t="s">
+      <c r="A14" s="10" t="s">
         <v>290</v>
       </c>
-      <c r="B14" s="14" t="s">
+      <c r="B14" s="10" t="s">
         <v>318</v>
       </c>
-      <c r="C14" s="14" t="s">
+      <c r="C14" s="10" t="s">
         <v>319</v>
       </c>
-      <c r="D14" s="14" t="s">
+      <c r="D14" s="10" t="s">
         <v>320</v>
       </c>
-      <c r="F14" s="14" t="s">
+      <c r="F14" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="G14" s="14" t="s">
+      <c r="G14" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="H14" s="14" t="s">
+      <c r="H14" s="10" t="s">
         <v>321</v>
       </c>
-      <c r="X14" s="23" t="s">
+      <c r="X14" s="19" t="s">
         <v>322</v>
       </c>
-      <c r="Y14" s="37">
+      <c r="Y14" s="33">
         <f t="shared" si="0"/>
         <v>3237.82</v>
       </c>
     </row>
     <row r="15" spans="1:25">
-      <c r="A15" s="25">
+      <c r="A15" s="21">
         <f>IF(AND('REPORTE CREDITOS DIARIOS'!A5&gt;=$A$5,'REPORTE CREDITOS DIARIOS'!A5&lt;=$C$5),'REPORTE CREDITOS DIARIOS'!A5,"")</f>
         <v>46235</v>
       </c>
-      <c r="B15" s="35">
+      <c r="B15" s="31">
         <f>IF(A15="",0,IF($E$5&lt;&gt;"TODAS",IFERROR(INDEX('REPORTE CREDITOS DIARIOS'!$B$5:$I$23,MATCH(A15,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,0),MATCH($E$5,'REPORTE CREDITOS DIARIOS'!$B$4:$I$4,0)),0),IF($G$5="TODOS",IFERROR(SUMIF('REPORTE CREDITOS DIARIOS'!$A$5:$A$23,A15,'REPORTE CREDITOS DIARIOS'!$J$5:$J$23),0),0)))</f>
         <v>9716.2900000000009</v>
       </c>
-      <c r="C15" s="35">
+      <c r="C15" s="31">
         <f>0</f>
         <v>0</v>
       </c>
-      <c r="D15" s="26">
+      <c r="D15" s="22">
         <f>IF(A15="",0,IF($G$5="TODOS",IFERROR(INDEX('REPORTE CREDITOS DIARIOS'!$K$5:$K$23,MATCH(A15,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,0)),0),IF(B15&gt;0,1,0)))</f>
         <v>4</v>
       </c>
-      <c r="F15" s="27" t="s">
+      <c r="F15" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="G15" s="28" t="s">
+      <c r="G15" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="H15" s="35">
+      <c r="H15" s="31">
         <f>IF(AND(OR($G$5="TODOS",TRIM($G$5)=TRIM(F15)),OR($E$5="TODAS",TEXT($E$5,"0")=TEXT(G15,"0"))),SUMIFS('REPORTE CREDITOS DIARIOS'!$B$5:$B$23,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,"&gt;="&amp;$A$5,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,"&lt;="&amp;$C$5),0)</f>
         <v>24450.060000000005</v>
       </c>
-      <c r="X15" s="23" t="s">
+      <c r="X15" s="19" t="s">
         <v>323</v>
       </c>
-      <c r="Y15" s="37">
+      <c r="Y15" s="33">
         <f t="shared" si="0"/>
         <v>11399.17</v>
       </c>
     </row>
     <row r="16" spans="1:25">
-      <c r="A16" s="29">
+      <c r="A16" s="25">
         <f>IF(AND('REPORTE CREDITOS DIARIOS'!A6&gt;=$A$5,'REPORTE CREDITOS DIARIOS'!A6&lt;=$C$5),'REPORTE CREDITOS DIARIOS'!A6,"")</f>
         <v>46236</v>
       </c>
-      <c r="B16" s="36">
+      <c r="B16" s="32">
         <f>IF(A16="",0,IF($E$5&lt;&gt;"TODAS",IFERROR(INDEX('REPORTE CREDITOS DIARIOS'!$B$5:$I$23,MATCH(A16,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,0),MATCH($E$5,'REPORTE CREDITOS DIARIOS'!$B$4:$I$4,0)),0),IF($G$5="TODOS",IFERROR(SUMIF('REPORTE CREDITOS DIARIOS'!$A$5:$A$23,A16,'REPORTE CREDITOS DIARIOS'!$J$5:$J$23),0),0)))</f>
         <v>0</v>
       </c>
-      <c r="C16" s="36">
+      <c r="C16" s="32">
         <f t="shared" ref="C16:C33" si="1">B16-B15</f>
         <v>-9716.2900000000009</v>
       </c>
-      <c r="D16" s="30">
+      <c r="D16" s="26">
         <f>IF(A16="",0,IF($G$5="TODOS",IFERROR(INDEX('REPORTE CREDITOS DIARIOS'!$K$5:$K$23,MATCH(A16,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,0)),0),IF(B16&gt;0,1,0)))</f>
         <v>0</v>
       </c>
-      <c r="F16" s="31" t="s">
+      <c r="F16" s="27" t="s">
         <v>289</v>
       </c>
-      <c r="G16" s="32" t="s">
+      <c r="G16" s="28" t="s">
         <v>9</v>
       </c>
-      <c r="H16" s="36">
+      <c r="H16" s="32">
         <f>IF(AND(OR($G$5="TODOS",TRIM($G$5)=TRIM(F16)),OR($E$5="TODAS",TEXT($E$5,"0")=TEXT(G16,"0"))),SUMIFS('REPORTE CREDITOS DIARIOS'!$C$5:$C$23,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,"&gt;="&amp;$A$5,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,"&lt;="&amp;$C$5),0)</f>
         <v>7792.46</v>
       </c>
-      <c r="X16" s="23" t="s">
+      <c r="X16" s="19" t="s">
         <v>324</v>
       </c>
-      <c r="Y16" s="37">
+      <c r="Y16" s="33">
         <f t="shared" si="0"/>
         <v>902.05</v>
       </c>
     </row>
     <row r="17" spans="1:25">
-      <c r="A17" s="25">
+      <c r="A17" s="21">
         <f>IF(AND('REPORTE CREDITOS DIARIOS'!A7&gt;=$A$5,'REPORTE CREDITOS DIARIOS'!A7&lt;=$C$5),'REPORTE CREDITOS DIARIOS'!A7,"")</f>
         <v>46237</v>
       </c>
-      <c r="B17" s="35">
+      <c r="B17" s="31">
         <f>IF(A17="",0,IF($E$5&lt;&gt;"TODAS",IFERROR(INDEX('REPORTE CREDITOS DIARIOS'!$B$5:$I$23,MATCH(A17,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,0),MATCH($E$5,'REPORTE CREDITOS DIARIOS'!$B$4:$I$4,0)),0),IF($G$5="TODOS",IFERROR(SUMIF('REPORTE CREDITOS DIARIOS'!$A$5:$A$23,A17,'REPORTE CREDITOS DIARIOS'!$J$5:$J$23),0),0)))</f>
         <v>2343.56</v>
       </c>
-      <c r="C17" s="35">
+      <c r="C17" s="31">
         <f t="shared" si="1"/>
         <v>2343.56</v>
       </c>
-      <c r="D17" s="26">
+      <c r="D17" s="22">
         <f>IF(A17="",0,IF($G$5="TODOS",IFERROR(INDEX('REPORTE CREDITOS DIARIOS'!$K$5:$K$23,MATCH(A17,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,0)),0),IF(B17&gt;0,1,0)))</f>
         <v>4</v>
       </c>
-      <c r="F17" s="27" t="s">
+      <c r="F17" s="23" t="s">
         <v>289</v>
       </c>
-      <c r="G17" s="28" t="s">
+      <c r="G17" s="24" t="s">
         <v>10</v>
       </c>
-      <c r="H17" s="35">
+      <c r="H17" s="31">
         <f>IF(AND(OR($G$5="TODOS",TRIM($G$5)=TRIM(F17)),OR($E$5="TODAS",TEXT($E$5,"0")=TEXT(G17,"0"))),SUMIFS('REPORTE CREDITOS DIARIOS'!$D$5:$D$23,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,"&gt;="&amp;$A$5,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,"&lt;="&amp;$C$5),0)</f>
         <v>4756.09</v>
       </c>
-      <c r="X17" s="23" t="s">
+      <c r="X17" s="19" t="s">
         <v>325</v>
       </c>
-      <c r="Y17" s="37">
+      <c r="Y17" s="33">
         <f t="shared" si="0"/>
         <v>519.84</v>
       </c>
     </row>
     <row r="18" spans="1:25">
-      <c r="A18" s="29">
+      <c r="A18" s="25">
         <f>IF(AND('REPORTE CREDITOS DIARIOS'!A8&gt;=$A$5,'REPORTE CREDITOS DIARIOS'!A8&lt;=$C$5),'REPORTE CREDITOS DIARIOS'!A8,"")</f>
         <v>46238</v>
       </c>
-      <c r="B18" s="36">
+      <c r="B18" s="32">
         <f>IF(A18="",0,IF($E$5&lt;&gt;"TODAS",IFERROR(INDEX('REPORTE CREDITOS DIARIOS'!$B$5:$I$23,MATCH(A18,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,0),MATCH($E$5,'REPORTE CREDITOS DIARIOS'!$B$4:$I$4,0)),0),IF($G$5="TODOS",IFERROR(SUMIF('REPORTE CREDITOS DIARIOS'!$A$5:$A$23,A18,'REPORTE CREDITOS DIARIOS'!$J$5:$J$23),0),0)))</f>
         <v>4295.79</v>
       </c>
-      <c r="C18" s="36">
+      <c r="C18" s="32">
         <f t="shared" si="1"/>
         <v>1952.23</v>
       </c>
-      <c r="D18" s="30">
+      <c r="D18" s="26">
         <f>IF(A18="",0,IF($G$5="TODOS",IFERROR(INDEX('REPORTE CREDITOS DIARIOS'!$K$5:$K$23,MATCH(A18,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,0)),0),IF(B18&gt;0,1,0)))</f>
         <v>7</v>
       </c>
-      <c r="F18" s="31" t="s">
+      <c r="F18" s="27" t="s">
         <v>130</v>
       </c>
-      <c r="G18" s="32" t="s">
+      <c r="G18" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="H18" s="36">
+      <c r="H18" s="32">
         <f>IF(AND(OR($G$5="TODOS",TRIM($G$5)=TRIM(F18)),OR($E$5="TODAS",TEXT($E$5,"0")=TEXT(G18,"0"))),SUMIFS('REPORTE CREDITOS DIARIOS'!$E$5:$E$23,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,"&gt;="&amp;$A$5,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,"&lt;="&amp;$C$5),0)</f>
         <v>9106.92</v>
       </c>
-      <c r="X18" s="23" t="s">
+      <c r="X18" s="19" t="s">
         <v>326</v>
       </c>
-      <c r="Y18" s="37">
+      <c r="Y18" s="33">
         <f t="shared" si="0"/>
         <v>3533.68</v>
       </c>
     </row>
     <row r="19" spans="1:25">
-      <c r="A19" s="25">
+      <c r="A19" s="21">
         <f>IF(AND('REPORTE CREDITOS DIARIOS'!A9&gt;=$A$5,'REPORTE CREDITOS DIARIOS'!A9&lt;=$C$5),'REPORTE CREDITOS DIARIOS'!A9,"")</f>
         <v>46239</v>
       </c>
-      <c r="B19" s="35">
+      <c r="B19" s="31">
         <f>IF(A19="",0,IF($E$5&lt;&gt;"TODAS",IFERROR(INDEX('REPORTE CREDITOS DIARIOS'!$B$5:$I$23,MATCH(A19,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,0),MATCH($E$5,'REPORTE CREDITOS DIARIOS'!$B$4:$I$4,0)),0),IF($G$5="TODOS",IFERROR(SUMIF('REPORTE CREDITOS DIARIOS'!$A$5:$A$23,A19,'REPORTE CREDITOS DIARIOS'!$J$5:$J$23),0),0)))</f>
         <v>1503.46</v>
       </c>
-      <c r="C19" s="35">
+      <c r="C19" s="31">
         <f t="shared" si="1"/>
         <v>-2792.33</v>
       </c>
-      <c r="D19" s="26">
+      <c r="D19" s="22">
         <f>IF(A19="",0,IF($G$5="TODOS",IFERROR(INDEX('REPORTE CREDITOS DIARIOS'!$K$5:$K$23,MATCH(A19,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,0)),0),IF(B19&gt;0,1,0)))</f>
         <v>5</v>
       </c>
-      <c r="F19" s="27" t="s">
+      <c r="F19" s="23" t="s">
         <v>130</v>
       </c>
-      <c r="G19" s="28" t="s">
+      <c r="G19" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="H19" s="35">
+      <c r="H19" s="31">
         <f>IF(AND(OR($G$5="TODOS",TRIM($G$5)=TRIM(F19)),OR($E$5="TODAS",TEXT($E$5,"0")=TEXT(G19,"0"))),SUMIFS('REPORTE CREDITOS DIARIOS'!$F$5:$F$23,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,"&gt;="&amp;$A$5,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,"&lt;="&amp;$C$5),0)</f>
         <v>18332.919999999998</v>
       </c>
-      <c r="X19" s="23" t="s">
+      <c r="X19" s="19" t="s">
         <v>327</v>
       </c>
-      <c r="Y19" s="37">
+      <c r="Y19" s="33">
         <f t="shared" si="0"/>
         <v>8791.41</v>
       </c>
     </row>
     <row r="20" spans="1:25">
-      <c r="A20" s="29">
+      <c r="A20" s="25">
         <f>IF(AND('REPORTE CREDITOS DIARIOS'!A10&gt;=$A$5,'REPORTE CREDITOS DIARIOS'!A10&lt;=$C$5),'REPORTE CREDITOS DIARIOS'!A10,"")</f>
         <v>46240</v>
       </c>
-      <c r="B20" s="36">
+      <c r="B20" s="32">
         <f>IF(A20="",0,IF($E$5&lt;&gt;"TODAS",IFERROR(INDEX('REPORTE CREDITOS DIARIOS'!$B$5:$I$23,MATCH(A20,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,0),MATCH($E$5,'REPORTE CREDITOS DIARIOS'!$B$4:$I$4,0)),0),IF($G$5="TODOS",IFERROR(SUMIF('REPORTE CREDITOS DIARIOS'!$A$5:$A$23,A20,'REPORTE CREDITOS DIARIOS'!$J$5:$J$23),0),0)))</f>
         <v>622.82000000000005</v>
       </c>
-      <c r="C20" s="36">
+      <c r="C20" s="32">
         <f t="shared" si="1"/>
         <v>-880.64</v>
       </c>
-      <c r="D20" s="30">
+      <c r="D20" s="26">
         <f>IF(A20="",0,IF($G$5="TODOS",IFERROR(INDEX('REPORTE CREDITOS DIARIOS'!$K$5:$K$23,MATCH(A20,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,0)),0),IF(B20&gt;0,1,0)))</f>
         <v>1</v>
       </c>
-      <c r="F20" s="31" t="s">
+      <c r="F20" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="G20" s="32" t="s">
+      <c r="G20" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="H20" s="36">
+      <c r="H20" s="32">
         <f>IF(AND(OR($G$5="TODOS",TRIM($G$5)=TRIM(F20)),OR($E$5="TODAS",TEXT($E$5,"0")=TEXT(G20,"0"))),SUMIFS('REPORTE CREDITOS DIARIOS'!$G$5:$G$23,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,"&gt;="&amp;$A$5,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,"&lt;="&amp;$C$5),0)</f>
         <v>5636.83</v>
       </c>
-      <c r="X20" s="23" t="s">
+      <c r="X20" s="19" t="s">
         <v>328</v>
       </c>
-      <c r="Y20" s="37">
+      <c r="Y20" s="33">
         <f t="shared" si="0"/>
         <v>8257.92</v>
       </c>
     </row>
     <row r="21" spans="1:25" ht="14.4">
-      <c r="A21" s="25">
+      <c r="A21" s="21">
         <f>IF(AND('REPORTE CREDITOS DIARIOS'!A11&gt;=$A$5,'REPORTE CREDITOS DIARIOS'!A11&lt;=$C$5),'REPORTE CREDITOS DIARIOS'!A11,"")</f>
         <v>46241</v>
       </c>
-      <c r="B21" s="35">
+      <c r="B21" s="31">
         <f>IF(A21="",0,IF($E$5&lt;&gt;"TODAS",IFERROR(INDEX('REPORTE CREDITOS DIARIOS'!$B$5:$I$23,MATCH(A21,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,0),MATCH($E$5,'REPORTE CREDITOS DIARIOS'!$B$4:$I$4,0)),0),IF($G$5="TODOS",IFERROR(SUMIF('REPORTE CREDITOS DIARIOS'!$A$5:$A$23,A21,'REPORTE CREDITOS DIARIOS'!$J$5:$J$23),0),0)))</f>
         <v>2766.44</v>
       </c>
-      <c r="C21" s="35">
+      <c r="C21" s="31">
         <f t="shared" si="1"/>
         <v>2143.62</v>
       </c>
-      <c r="D21" s="26">
+      <c r="D21" s="22">
         <f>IF(A21="",0,IF($G$5="TODOS",IFERROR(INDEX('REPORTE CREDITOS DIARIOS'!$K$5:$K$23,MATCH(A21,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,0)),0),IF(B21&gt;0,1,0)))</f>
         <v>6</v>
       </c>
-      <c r="F21" s="27" t="s">
+      <c r="F21" s="23" t="s">
         <v>241</v>
       </c>
-      <c r="G21" s="28" t="s">
+      <c r="G21" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="H21" s="35">
+      <c r="H21" s="31">
         <f>IF(AND(OR($G$5="TODOS",TRIM($G$5)=TRIM(F21)),OR($E$5="TODAS",TEXT($E$5,"0")=TEXT(G21,"0"))),SUMIFS('REPORTE CREDITOS DIARIOS'!$H$5:$H$23,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,"&gt;="&amp;$A$5,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,"&lt;="&amp;$C$5),0)</f>
         <v>32704.7</v>
       </c>
-      <c r="Y21" s="33"/>
+      <c r="Y21" s="29"/>
     </row>
     <row r="22" spans="1:25" ht="14.4">
-      <c r="A22" s="29">
+      <c r="A22" s="25">
         <f>IF(AND('REPORTE CREDITOS DIARIOS'!A12&gt;=$A$5,'REPORTE CREDITOS DIARIOS'!A12&lt;=$C$5),'REPORTE CREDITOS DIARIOS'!A12,"")</f>
         <v>46242</v>
       </c>
-      <c r="B22" s="36">
+      <c r="B22" s="32">
         <f>IF(A22="",0,IF($E$5&lt;&gt;"TODAS",IFERROR(INDEX('REPORTE CREDITOS DIARIOS'!$B$5:$I$23,MATCH(A22,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,0),MATCH($E$5,'REPORTE CREDITOS DIARIOS'!$B$4:$I$4,0)),0),IF($G$5="TODOS",IFERROR(SUMIF('REPORTE CREDITOS DIARIOS'!$A$5:$A$23,A22,'REPORTE CREDITOS DIARIOS'!$J$5:$J$23),0),0)))</f>
         <v>814.73</v>
       </c>
-      <c r="C22" s="36">
+      <c r="C22" s="32">
         <f t="shared" si="1"/>
         <v>-1951.71</v>
       </c>
-      <c r="D22" s="30">
+      <c r="D22" s="26">
         <f>IF(A22="",0,IF($G$5="TODOS",IFERROR(INDEX('REPORTE CREDITOS DIARIOS'!$K$5:$K$23,MATCH(A22,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,0)),0),IF(B22&gt;0,1,0)))</f>
         <v>1</v>
       </c>
-      <c r="F22" s="31" t="s">
+      <c r="F22" s="27" t="s">
         <v>241</v>
       </c>
-      <c r="G22" s="32" t="s">
+      <c r="G22" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="H22" s="36">
+      <c r="H22" s="32">
         <f>IF(AND(OR($G$5="TODOS",TRIM($G$5)=TRIM(F22)),OR($E$5="TODAS",TEXT($E$5,"0")=TEXT(G22,"0"))),SUMIFS('REPORTE CREDITOS DIARIOS'!$I$5:$I$23,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,"&gt;="&amp;$A$5,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,"&lt;="&amp;$C$5),0)</f>
         <v>101.91</v>
       </c>
-      <c r="Y22" s="33"/>
+      <c r="Y22" s="29"/>
     </row>
     <row r="23" spans="1:25" ht="14.4">
-      <c r="A23" s="25">
+      <c r="A23" s="21">
         <f>IF(AND('REPORTE CREDITOS DIARIOS'!A13&gt;=$A$5,'REPORTE CREDITOS DIARIOS'!A13&lt;=$C$5),'REPORTE CREDITOS DIARIOS'!A13,"")</f>
         <v>46243</v>
       </c>
-      <c r="B23" s="35">
+      <c r="B23" s="31">
         <f>IF(A23="",0,IF($E$5&lt;&gt;"TODAS",IFERROR(INDEX('REPORTE CREDITOS DIARIOS'!$B$5:$I$23,MATCH(A23,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,0),MATCH($E$5,'REPORTE CREDITOS DIARIOS'!$B$4:$I$4,0)),0),IF($G$5="TODOS",IFERROR(SUMIF('REPORTE CREDITOS DIARIOS'!$A$5:$A$23,A23,'REPORTE CREDITOS DIARIOS'!$J$5:$J$23),0),0)))</f>
         <v>0</v>
       </c>
-      <c r="C23" s="35">
+      <c r="C23" s="31">
         <f t="shared" si="1"/>
         <v>-814.73</v>
       </c>
-      <c r="D23" s="26">
+      <c r="D23" s="22">
         <f>IF(A23="",0,IF($G$5="TODOS",IFERROR(INDEX('REPORTE CREDITOS DIARIOS'!$K$5:$K$23,MATCH(A23,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,0)),0),IF(B23&gt;0,1,0)))</f>
         <v>0</v>
       </c>
-      <c r="F23" s="52" t="s">
-        <v>331</v>
-      </c>
-      <c r="G23" s="52"/>
-      <c r="H23" s="34">
+      <c r="F23" s="43" t="s">
+        <v>329</v>
+      </c>
+      <c r="G23" s="43"/>
+      <c r="H23" s="30">
         <f>SUM(H15:H22)</f>
         <v>102881.89</v>
       </c>
-      <c r="Y23" s="33"/>
+      <c r="Y23" s="29"/>
     </row>
     <row r="24" spans="1:25" ht="14.4">
-      <c r="A24" s="29">
+      <c r="A24" s="25">
         <f>IF(AND('REPORTE CREDITOS DIARIOS'!A14&gt;=$A$5,'REPORTE CREDITOS DIARIOS'!A14&lt;=$C$5),'REPORTE CREDITOS DIARIOS'!A14,"")</f>
         <v>46244</v>
       </c>
-      <c r="B24" s="36">
+      <c r="B24" s="32">
         <f>IF(A24="",0,IF($E$5&lt;&gt;"TODAS",IFERROR(INDEX('REPORTE CREDITOS DIARIOS'!$B$5:$I$23,MATCH(A24,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,0),MATCH($E$5,'REPORTE CREDITOS DIARIOS'!$B$4:$I$4,0)),0),IF($G$5="TODOS",IFERROR(SUMIF('REPORTE CREDITOS DIARIOS'!$A$5:$A$23,A24,'REPORTE CREDITOS DIARIOS'!$J$5:$J$23),0),0)))</f>
         <v>2835.55</v>
       </c>
-      <c r="C24" s="36">
+      <c r="C24" s="32">
         <f t="shared" si="1"/>
         <v>2835.55</v>
       </c>
-      <c r="D24" s="30">
+      <c r="D24" s="26">
         <f>IF(A24="",0,IF($G$5="TODOS",IFERROR(INDEX('REPORTE CREDITOS DIARIOS'!$K$5:$K$23,MATCH(A24,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,0)),0),IF(B24&gt;0,1,0)))</f>
         <v>7</v>
       </c>
-      <c r="Y24" s="33"/>
+      <c r="Y24" s="29"/>
     </row>
     <row r="25" spans="1:25" ht="14.4">
-      <c r="A25" s="25">
+      <c r="A25" s="21">
         <f>IF(AND('REPORTE CREDITOS DIARIOS'!A15&gt;=$A$5,'REPORTE CREDITOS DIARIOS'!A15&lt;=$C$5),'REPORTE CREDITOS DIARIOS'!A15,"")</f>
         <v>46245</v>
       </c>
-      <c r="B25" s="35">
+      <c r="B25" s="31">
         <f>IF(A25="",0,IF($E$5&lt;&gt;"TODAS",IFERROR(INDEX('REPORTE CREDITOS DIARIOS'!$B$5:$I$23,MATCH(A25,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,0),MATCH($E$5,'REPORTE CREDITOS DIARIOS'!$B$4:$I$4,0)),0),IF($G$5="TODOS",IFERROR(SUMIF('REPORTE CREDITOS DIARIOS'!$A$5:$A$23,A25,'REPORTE CREDITOS DIARIOS'!$J$5:$J$23),0),0)))</f>
         <v>32978.11</v>
       </c>
-      <c r="C25" s="35">
+      <c r="C25" s="31">
         <f t="shared" si="1"/>
         <v>30142.560000000001</v>
       </c>
-      <c r="D25" s="26">
+      <c r="D25" s="22">
         <f>IF(A25="",0,IF($G$5="TODOS",IFERROR(INDEX('REPORTE CREDITOS DIARIOS'!$K$5:$K$23,MATCH(A25,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,0)),0),IF(B25&gt;0,1,0)))</f>
         <v>6</v>
       </c>
-      <c r="Y25" s="33"/>
+      <c r="Y25" s="29"/>
     </row>
     <row r="26" spans="1:25" ht="14.4">
-      <c r="A26" s="29">
+      <c r="A26" s="25">
         <f>IF(AND('REPORTE CREDITOS DIARIOS'!A16&gt;=$A$5,'REPORTE CREDITOS DIARIOS'!A16&lt;=$C$5),'REPORTE CREDITOS DIARIOS'!A16,"")</f>
         <v>46246</v>
       </c>
-      <c r="B26" s="36">
+      <c r="B26" s="32">
         <f>IF(A26="",0,IF($E$5&lt;&gt;"TODAS",IFERROR(INDEX('REPORTE CREDITOS DIARIOS'!$B$5:$I$23,MATCH(A26,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,0),MATCH($E$5,'REPORTE CREDITOS DIARIOS'!$B$4:$I$4,0)),0),IF($G$5="TODOS",IFERROR(SUMIF('REPORTE CREDITOS DIARIOS'!$A$5:$A$23,A26,'REPORTE CREDITOS DIARIOS'!$J$5:$J$23),0),0)))</f>
         <v>8363.25</v>
       </c>
-      <c r="C26" s="36">
+      <c r="C26" s="32">
         <f t="shared" si="1"/>
         <v>-24614.86</v>
       </c>
-      <c r="D26" s="30">
+      <c r="D26" s="26">
         <f>IF(A26="",0,IF($G$5="TODOS",IFERROR(INDEX('REPORTE CREDITOS DIARIOS'!$K$5:$K$23,MATCH(A26,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,0)),0),IF(B26&gt;0,1,0)))</f>
         <v>6</v>
       </c>
-      <c r="Y26" s="33"/>
+      <c r="Y26" s="29"/>
     </row>
     <row r="27" spans="1:25" ht="14.4">
-      <c r="A27" s="25">
+      <c r="A27" s="21">
         <f>IF(AND('REPORTE CREDITOS DIARIOS'!A17&gt;=$A$5,'REPORTE CREDITOS DIARIOS'!A17&lt;=$C$5),'REPORTE CREDITOS DIARIOS'!A17,"")</f>
         <v>46247</v>
       </c>
-      <c r="B27" s="35">
+      <c r="B27" s="31">
         <f>IF(A27="",0,IF($E$5&lt;&gt;"TODAS",IFERROR(INDEX('REPORTE CREDITOS DIARIOS'!$B$5:$I$23,MATCH(A27,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,0),MATCH($E$5,'REPORTE CREDITOS DIARIOS'!$B$4:$I$4,0)),0),IF($G$5="TODOS",IFERROR(SUMIF('REPORTE CREDITOS DIARIOS'!$A$5:$A$23,A27,'REPORTE CREDITOS DIARIOS'!$J$5:$J$23),0),0)))</f>
         <v>3237.82</v>
       </c>
-      <c r="C27" s="35">
+      <c r="C27" s="31">
         <f t="shared" si="1"/>
         <v>-5125.43</v>
       </c>
-      <c r="D27" s="26">
+      <c r="D27" s="22">
         <f>IF(A27="",0,IF($G$5="TODOS",IFERROR(INDEX('REPORTE CREDITOS DIARIOS'!$K$5:$K$23,MATCH(A27,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,0)),0),IF(B27&gt;0,1,0)))</f>
         <v>6</v>
       </c>
-      <c r="Y27" s="33"/>
+      <c r="Y27" s="29"/>
     </row>
     <row r="28" spans="1:25" ht="14.4">
-      <c r="A28" s="29">
+      <c r="A28" s="25">
         <f>IF(AND('REPORTE CREDITOS DIARIOS'!A18&gt;=$A$5,'REPORTE CREDITOS DIARIOS'!A18&lt;=$C$5),'REPORTE CREDITOS DIARIOS'!A18,"")</f>
         <v>46248</v>
       </c>
-      <c r="B28" s="36">
+      <c r="B28" s="32">
         <f>IF(A28="",0,IF($E$5&lt;&gt;"TODAS",IFERROR(INDEX('REPORTE CREDITOS DIARIOS'!$B$5:$I$23,MATCH(A28,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,0),MATCH($E$5,'REPORTE CREDITOS DIARIOS'!$B$4:$I$4,0)),0),IF($G$5="TODOS",IFERROR(SUMIF('REPORTE CREDITOS DIARIOS'!$A$5:$A$23,A28,'REPORTE CREDITOS DIARIOS'!$J$5:$J$23),0),0)))</f>
         <v>11399.17</v>
       </c>
-      <c r="C28" s="36">
+      <c r="C28" s="32">
         <f t="shared" si="1"/>
         <v>8161.35</v>
       </c>
-      <c r="D28" s="30">
+      <c r="D28" s="26">
         <f>IF(A28="",0,IF($G$5="TODOS",IFERROR(INDEX('REPORTE CREDITOS DIARIOS'!$K$5:$K$23,MATCH(A28,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,0)),0),IF(B28&gt;0,1,0)))</f>
         <v>5</v>
       </c>
-      <c r="Y28" s="33"/>
+      <c r="Y28" s="29"/>
     </row>
     <row r="29" spans="1:25" ht="14.4">
-      <c r="A29" s="25">
+      <c r="A29" s="21">
         <f>IF(AND('REPORTE CREDITOS DIARIOS'!A19&gt;=$A$5,'REPORTE CREDITOS DIARIOS'!A19&lt;=$C$5),'REPORTE CREDITOS DIARIOS'!A19,"")</f>
         <v>46249</v>
       </c>
-      <c r="B29" s="35">
+      <c r="B29" s="31">
         <f>IF(A29="",0,IF($E$5&lt;&gt;"TODAS",IFERROR(INDEX('REPORTE CREDITOS DIARIOS'!$B$5:$I$23,MATCH(A29,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,0),MATCH($E$5,'REPORTE CREDITOS DIARIOS'!$B$4:$I$4,0)),0),IF($G$5="TODOS",IFERROR(SUMIF('REPORTE CREDITOS DIARIOS'!$A$5:$A$23,A29,'REPORTE CREDITOS DIARIOS'!$J$5:$J$23),0),0)))</f>
         <v>902.05</v>
       </c>
-      <c r="C29" s="35">
+      <c r="C29" s="31">
         <f t="shared" si="1"/>
         <v>-10497.12</v>
       </c>
-      <c r="D29" s="26">
+      <c r="D29" s="22">
         <f>IF(A29="",0,IF($G$5="TODOS",IFERROR(INDEX('REPORTE CREDITOS DIARIOS'!$K$5:$K$23,MATCH(A29,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,0)),0),IF(B29&gt;0,1,0)))</f>
         <v>4</v>
       </c>
-      <c r="Y29" s="33"/>
+      <c r="Y29" s="29"/>
     </row>
     <row r="30" spans="1:25" ht="14.4">
-      <c r="A30" s="29">
+      <c r="A30" s="25">
         <f>IF(AND('REPORTE CREDITOS DIARIOS'!A20&gt;=$A$5,'REPORTE CREDITOS DIARIOS'!A20&lt;=$C$5),'REPORTE CREDITOS DIARIOS'!A20,"")</f>
         <v>46250</v>
       </c>
-      <c r="B30" s="36">
+      <c r="B30" s="32">
         <f>IF(A30="",0,IF($E$5&lt;&gt;"TODAS",IFERROR(INDEX('REPORTE CREDITOS DIARIOS'!$B$5:$I$23,MATCH(A30,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,0),MATCH($E$5,'REPORTE CREDITOS DIARIOS'!$B$4:$I$4,0)),0),IF($G$5="TODOS",IFERROR(SUMIF('REPORTE CREDITOS DIARIOS'!$A$5:$A$23,A30,'REPORTE CREDITOS DIARIOS'!$J$5:$J$23),0),0)))</f>
         <v>519.84</v>
       </c>
-      <c r="C30" s="36">
+      <c r="C30" s="32">
         <f t="shared" si="1"/>
         <v>-382.20999999999992</v>
       </c>
-      <c r="D30" s="30">
+      <c r="D30" s="26">
         <f>IF(A30="",0,IF($G$5="TODOS",IFERROR(INDEX('REPORTE CREDITOS DIARIOS'!$K$5:$K$23,MATCH(A30,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,0)),0),IF(B30&gt;0,1,0)))</f>
         <v>2</v>
       </c>
-      <c r="Y30" s="33"/>
+      <c r="Y30" s="29"/>
     </row>
     <row r="31" spans="1:25" ht="14.4">
-      <c r="A31" s="25">
+      <c r="A31" s="21">
         <f>IF(AND('REPORTE CREDITOS DIARIOS'!A21&gt;=$A$5,'REPORTE CREDITOS DIARIOS'!A21&lt;=$C$5),'REPORTE CREDITOS DIARIOS'!A21,"")</f>
         <v>46251</v>
       </c>
-      <c r="B31" s="35">
+      <c r="B31" s="31">
         <f>IF(A31="",0,IF($E$5&lt;&gt;"TODAS",IFERROR(INDEX('REPORTE CREDITOS DIARIOS'!$B$5:$I$23,MATCH(A31,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,0),MATCH($E$5,'REPORTE CREDITOS DIARIOS'!$B$4:$I$4,0)),0),IF($G$5="TODOS",IFERROR(SUMIF('REPORTE CREDITOS DIARIOS'!$A$5:$A$23,A31,'REPORTE CREDITOS DIARIOS'!$J$5:$J$23),0),0)))</f>
         <v>3533.68</v>
       </c>
-      <c r="C31" s="35">
+      <c r="C31" s="31">
         <f t="shared" si="1"/>
         <v>3013.8399999999997</v>
       </c>
-      <c r="D31" s="26">
+      <c r="D31" s="22">
         <f>IF(A31="",0,IF($G$5="TODOS",IFERROR(INDEX('REPORTE CREDITOS DIARIOS'!$K$5:$K$23,MATCH(A31,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,0)),0),IF(B31&gt;0,1,0)))</f>
         <v>6</v>
       </c>
-      <c r="Y31" s="33"/>
+      <c r="Y31" s="29"/>
     </row>
     <row r="32" spans="1:25" ht="14.4">
-      <c r="A32" s="29">
+      <c r="A32" s="25">
         <f>IF(AND('REPORTE CREDITOS DIARIOS'!A22&gt;=$A$5,'REPORTE CREDITOS DIARIOS'!A22&lt;=$C$5),'REPORTE CREDITOS DIARIOS'!A22,"")</f>
         <v>46252</v>
       </c>
-      <c r="B32" s="36">
+      <c r="B32" s="32">
         <f>IF(A32="",0,IF($E$5&lt;&gt;"TODAS",IFERROR(INDEX('REPORTE CREDITOS DIARIOS'!$B$5:$I$23,MATCH(A32,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,0),MATCH($E$5,'REPORTE CREDITOS DIARIOS'!$B$4:$I$4,0)),0),IF($G$5="TODOS",IFERROR(SUMIF('REPORTE CREDITOS DIARIOS'!$A$5:$A$23,A32,'REPORTE CREDITOS DIARIOS'!$J$5:$J$23),0),0)))</f>
         <v>8791.41</v>
       </c>
-      <c r="C32" s="36">
+      <c r="C32" s="32">
         <f t="shared" si="1"/>
         <v>5257.73</v>
       </c>
-      <c r="D32" s="30">
+      <c r="D32" s="26">
         <f>IF(A32="",0,IF($G$5="TODOS",IFERROR(INDEX('REPORTE CREDITOS DIARIOS'!$K$5:$K$23,MATCH(A32,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,0)),0),IF(B32&gt;0,1,0)))</f>
         <v>5</v>
       </c>
-      <c r="Y32" s="33"/>
+      <c r="Y32" s="29"/>
     </row>
     <row r="33" spans="1:25" ht="14.4">
-      <c r="A33" s="25">
+      <c r="A33" s="21">
         <f>IF(AND('REPORTE CREDITOS DIARIOS'!A23&gt;=$A$5,'REPORTE CREDITOS DIARIOS'!A23&lt;=$C$5),'REPORTE CREDITOS DIARIOS'!A23,"")</f>
         <v>46253</v>
       </c>
-      <c r="B33" s="35">
+      <c r="B33" s="31">
         <f>IF(A33="",0,IF($E$5&lt;&gt;"TODAS",IFERROR(INDEX('REPORTE CREDITOS DIARIOS'!$B$5:$I$23,MATCH(A33,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,0),MATCH($E$5,'REPORTE CREDITOS DIARIOS'!$B$4:$I$4,0)),0),IF($G$5="TODOS",IFERROR(SUMIF('REPORTE CREDITOS DIARIOS'!$A$5:$A$23,A33,'REPORTE CREDITOS DIARIOS'!$J$5:$J$23),0),0)))</f>
         <v>8257.92</v>
       </c>
-      <c r="C33" s="35">
+      <c r="C33" s="31">
         <f t="shared" si="1"/>
         <v>-533.48999999999978</v>
       </c>
-      <c r="D33" s="26">
+      <c r="D33" s="22">
         <f>IF(A33="",0,IF($G$5="TODOS",IFERROR(INDEX('REPORTE CREDITOS DIARIOS'!$K$5:$K$23,MATCH(A33,'REPORTE CREDITOS DIARIOS'!$A$5:$A$23,0)),0),IF(B33&gt;0,1,0)))</f>
         <v>5</v>
       </c>
-      <c r="Y33" s="33"/>
+      <c r="Y33" s="29"/>
     </row>
     <row r="34" spans="1:25" ht="14.4">
-      <c r="Y34" s="33"/>
+      <c r="Y34" s="29"/>
     </row>
     <row r="35" spans="1:25" ht="14.4">
-      <c r="A35" s="42" t="s">
-        <v>329</v>
-      </c>
-      <c r="B35" s="39"/>
-      <c r="C35" s="39"/>
-      <c r="D35" s="39"/>
-      <c r="E35" s="39"/>
-      <c r="F35" s="39"/>
-      <c r="G35" s="39"/>
-      <c r="H35" s="39"/>
-      <c r="Y35" s="33"/>
+      <c r="A35" s="39" t="s">
+        <v>330</v>
+      </c>
+      <c r="B35" s="36"/>
+      <c r="C35" s="36"/>
+      <c r="D35" s="36"/>
+      <c r="E35" s="36"/>
+      <c r="F35" s="36"/>
+      <c r="G35" s="36"/>
+      <c r="H35" s="36"/>
+      <c r="Y35" s="29"/>
     </row>
   </sheetData>
-  <mergeCells count="16">
+  <mergeCells count="18">
+    <mergeCell ref="K7:L7"/>
+    <mergeCell ref="K8:L8"/>
+    <mergeCell ref="A35:H35"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="A13:D13"/>
+    <mergeCell ref="F13:H13"/>
     <mergeCell ref="I7:J7"/>
     <mergeCell ref="I8:J8"/>
     <mergeCell ref="F23:G23"/>
@@ -8554,13 +9333,6 @@
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="E5:F5"/>
     <mergeCell ref="G5:H5"/>
-    <mergeCell ref="A35:H35"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="E8:F8"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="A13:D13"/>
-    <mergeCell ref="F13:H13"/>
   </mergeCells>
   <conditionalFormatting sqref="H15:H22">
     <cfRule type="dataBar" priority="1">

</xml_diff>